<commit_message>
Make dedup_index filename compatible; save which records were detected as duplicates
</commit_message>
<xml_diff>
--- a/outputs/basic-processing/basic-exclusions/psycinfo-exclusions.xlsx
+++ b/outputs/basic-processing/basic-exclusions/psycinfo-exclusions.xlsx
@@ -36,13 +36,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="commentary-pub-types" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="commentary-title" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="methodology" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systematic review-pub-types" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systematic review-title" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systematic review-journal" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cohort profile" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="case report or case series-pub-" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="case report or case series-titl" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="case report or case series-jour" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reprint" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systematic review-pub-types" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systematic review-title" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="systematic review-journal" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cohort profile" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="case report or case series-pub-" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="case report or case series-titl" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="case report or case series-jour" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -582,7 +583,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>pregnancycomplicationsfollowingprenatalexposuretossrisormaternalpsychiatricdisorders:resultsfrompopulation-basednationalregisterdata;2015;malm</t>
+          <t>pregnancycomplicationsfollowingprenatalexposuretossrisormaternalpsychiatricdisordersresultsfrompopulationbasednationalregisterdata2015malm</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1958,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>aquasi-experimentaleffectivenessevaluationofthe'incredibleyearstoddler'parentingprogrammeonchildren'sdevelopmentaged5:astudyprotocol;2023;mooney</t>
+          <t>aquasiexperimentaleffectivenessevaluationoftheincredibleyearstoddlerparentingprogrammeonchildrensdevelopmentaged5astudyprotocol2023mooney</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2087,7 +2088,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>correctionto:associationofmaternalprenataldepressionandanxietywithtoddlersleep:thechina-anhuibirthcohortstudy;2022;ma</t>
+          <t>correctiontoassociationofmaternalprenataldepressionandanxietywithtoddlersleepthechinaanhuibirthcohortstudy2022ma</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2145,7 +2146,7 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>correctionto:perinatalhealthinamazontripleborderregion:cross-sectionalanalysiscomparingoutcomesinthebrazilian,peruvianandcolombianpopulation;2023;teixeira</t>
+          <t>correctiontoperinatalhealthinamazontripleborderregioncrosssectionalanalysiscomparingoutcomesinthebrazilianperuvianandcolombianpopulation2023teixeira</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2203,7 +2204,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>'associationofmaternaleatingdisorderswithpregnancyandneonataloutcomes':correction;2020;mantel</t>
+          <t>associationofmaternaleatingdisorderswithpregnancyandneonataloutcomescorrection2020mantel</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2259,7 +2260,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>cesareandeliveryundergeneralanesthesiacausingautisticspectrumdisorders:notverylikely;2020;raz</t>
+          <t>cesareandeliveryundergeneralanesthesiacausingautisticspectrumdisordersnotverylikely2020raz</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2317,7 +2318,7 @@
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>correctionto:predictingriskforearlybreastfeedingcessationinisrael;2022;gabay</t>
+          <t>correctiontopredictingriskforearlybreastfeedingcessationinisrael2022gabay</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2373,7 +2374,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>'changesinratesofinpatientpostpartumlong-actingreversiblecontraceptionandsterilizationintheusa,2012-2016':correction;2021;sheyn</t>
+          <t>changesinratesofinpatientpostpartumlongactingreversiblecontraceptionandsterilizationintheusa20122016correction2021sheyn</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2431,7 +2432,7 @@
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>long-termsurvivalinapatientwithmuscle-eye-braindisease;2015;falsaperla</t>
+          <t>longtermsurvivalinapatientwithmuscleeyebraindisease2015falsaperla</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2489,7 +2490,7 @@
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>whynotinduceeveryoneat39weeks?;2017;glantz</t>
+          <t>whynotinduceeveryoneat39weeks2017glantz</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2547,7 +2548,7 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>risksduringpregnancyinwomenwithepilepsy;2015;meador</t>
+          <t>risksduringpregnancyinwomenwithepilepsy2015meador</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2605,7 +2606,7 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>tokophobia,thefearofchildbirth,andthedecisiontobreastfeed;2015;kaymaz</t>
+          <t>tokophobiathefearofchildbirthandthedecisiontobreastfeed2015kaymaz</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2661,7 +2662,7 @@
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>'narcolepsyandpregnancy:aretrospectiveeuropeanevaluationof249pregnancies:'corrigendum;2014;maurovich-horvat</t>
+          <t>narcolepsyandpregnancyaretrospectiveeuropeanevaluationof249pregnanciescorrigendum2014maurovichhorvat</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2717,7 +2718,7 @@
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>continuationversusdiscontinuationoflithiumduringpregnancy:aretrospectivecaseseries;2014;deiana</t>
+          <t>continuationversusdiscontinuationoflithiumduringpregnancyaretrospectivecaseseries2014deiana</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2775,7 +2776,7 @@
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>maternalantidepressantuseandpersistentpulmonaryhypertensionofthenewborn;2015;giannakopoulos</t>
+          <t>maternalantidepressantuseandpersistentpulmonaryhypertensionofthenewborn2015giannakopoulos</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2833,7 +2834,7 @@
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>womenwithepilepsy;2016;sharma</t>
+          <t>womenwithepilepsy2016sharma</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2885,7 +2886,7 @@
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>'symptomsofeatingdisordersandfeedingpracticesinobesemothers':corrigendum;2014;zanardo</t>
+          <t>symptomsofeatingdisordersandfeedingpracticesinobesemotherscorrigendum2014zanardo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2941,7 +2942,7 @@
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>'maternalantidepressantuseandpersistentpulmonaryhypertensionofthenewborn':inreply;2015;huybrechts</t>
+          <t>maternalantidepressantuseandpersistentpulmonaryhypertensionofthenewborninreply2015huybrechts</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2999,7 +3000,7 @@
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
-          <t>'astudyofpostpartumdepressionandmaternalriskfactorsinqatar':corrigendum;2015;burgut</t>
+          <t>astudyofpostpartumdepressionandmaternalriskfactorsinqatarcorrigendum2015burgut</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3369,7 +3370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3431,1264 +3432,6 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>first_author_surname</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>prenatalpsychologicaldistressand11b-hsd2geneexpressioninhumanplacentas:systematicreviewandmeta-analysis;2024;tartour</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>prenatal psychological distress and 11b-hsd2 gene expression in human placentas: systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Tartour, Angham, Ibrahim;Chivese, Tawanda;Eltayeb, Safa;Elamin, Fatima, M.;Fthenou, Eleni;Seed Ahmed, Mohammed;Babu, Giridhara, Rathnaiah</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Background: The placenta acts as a buffer to regulate the degree of fetal exposure to maternal cortisol through the 11-Beta Hydroxysteroid Dehydrogenase isoenzyme type 2 (11-b HSD2) enzyme. We conducted a systematic review and meta-analysis to assess the effect of prenatal psychological distress (PPD) on placental 11-b HSD2 gene expression and explore the related mechanistic pathways involved in fetal neurodevelopment. Methods: We searched PubMed, Embase, Scopus, APA PsycInfo(r), and ProQuest Dissertations for observational studies assessing the association between PPD and 11-b HSD2 expression in human placentas. Adjusted regression coefficients (b) and corresponding 95% confidence intervals (CIs) were pooled based on three contextual PPD exposure groups: prenatal depression, anxiety symptoms, and perceived stress. Results: Of 3159 retrieved records, sixteen longitudinal studies involving 1869 participants across seven countries were included. Overall, exposure to PPD disorders showed weak negative associations with the placental 11-b HSD2 gene expression as follows: prenatal depression (b -0.01, 95% CI 0.05-0.02, I2=0%), anxiety symptoms (b -0.02, 95% CI 0.06-0.01, I2=0%), and perceived stress (b -0.01 95% CI 0.06-0.04, I2=62.8%). Third-trimester PPD exposure was more frequently associated with lower placental 11-b HSD2 levels. PPD and placental 11-b HSD2 were associated with changes in cortisol reactivity and the development of adverse health outcomes in mothers and children. Female-offspring were more vulnerable to PPD exposures. Conclusion: The study presents evidence of a modest role of prenatal psychological distress in regulating placental 11-b HSD2 gene expression. Future prospective cohorts utilizing larger sample sizes or advanced statistical methods to enhance the detection of small effect sizes should be planned. Additionally, controlling for key predictors such as the mother's ethnicity, trimester of PPD exposure, mode of delivery, and infant sex is crucial for valid exploration of PPD effects on fetal programming. (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10.1016/j.psyneuen.2024.107060</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Psychoneuroendocrinology</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Tartour</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>maternaloutcomesusingdelayedpushingversusimmediatepushinginthesecondstageoflabour:anumbrellareview;2024;deusa-lopez</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>maternal outcomes using delayed pushing versus immediate pushing in the second stage of labour: an umbrella review</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Deusa-Lopez, Paula;Cuenca-Martinez, Ferran;Sanchez-Martinez, Vanessa;Sempere-Rubio, Nuria</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Introduction: Different systematic reviews have been developed in the last decades about maternal risks of immediate pushing and delayed pushing, depending on the duration of the second stage of labour, but they do not provide conclusive evidence. Aim: The main aim of this overview of systematic reviews was to assess the maternal outcomes using delayed pushing and immediate pushing in the second stage of labour in women receiving epidural analgesia. Methods: We searched systematically in PubMed (Medline), EMBASE, CINAHL, and Scopus (October 26th, 2023). Methodological quality was analysed using AMSTAR and ROBIS scales, and the strength of evidence was established according to the guidelines advisory committee grading criteria. The outcome measures were the duration of the second stage of labour, duration of active pushing, caesarean section, instrumental vaginal birth, spontaneous vaginal birth, fatigue score, perineal lacerations, postpartum haemorrhage, and rate of episiotomy. Seven systematic reviews with and without meta-analysis were included. Results: Results showed that delayed pushing increases the total time of the second stage of labour, although delayed pushing decreases the duration of active pushing with moderate quality of evidence. Mixed results were found with respect to the variables instrumental vaginal birth, spontaneous vaginal birth, and fatigue score although the results favour delayed pushing or show no statistically significant differences with respect to immediate pushing. No favourable results were ever found for immediate pushing with respect to delayed pushing, with a limited quality of evidence. Even so, delayed pushing seems to be associated with a significant increase in spontaneous vaginal birth rates. The results found no significant differences between the immediate pushing and delayed pushing groups in the caesarean section rates, perineal lacerations, postpartum haemorrhage, and episiotomy ratio, with a limited quality of evidence. Conclusions: This study shows that delayed pushing during the second stage of labour produces at least the same maternal outcomes as immediate pushing, although we note that delayed pushing produces an increase of the duration of the second stage of labour, a shorter duration of the active pushing and a tendency to increase spontaneous vaginal birth and to reduce the instrumental vaginal birth rates and fatigue scores. This should be considered clinically. This review was registered in the International Prospective Register of Systematic Reviews PROSPERO (CRD42023397616). (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>10.1016/j.ijnurstu.2024.104693</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>International Journal of Nursing Studies</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Deusa-Lopez</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>theimpactoftelehealthapplicationsonpregnancyoutcomesandcostsinhigh-riskpregnancy:asystematicreviewandmeta-analysis;2024;gunesozturk</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>the impact of telehealth applications on pregnancy outcomes and costs in high-risk pregnancy: a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Gunes Ozturk, Gizem;Akyildiz, Deniz;Karacam, Zekiye</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Introduction: Telehealth is an applicable, acceptable, cost-effective, easily accessible, and speedy method for pregnant women. This study aimed to examine the impact of telehealth applications on pregnancy outcomes and costs in highrisk pregnancies. Methods: Studies were selected from PubMed, Science Direct, Web of Science, EBSCO, Scopus, and Clinical Key databases according to the inclusion and exclusion criteria from January to February 2021. Cochrane risk-of-bias tools were used in the quality assessment of the studies. Results: Four observational and eight randomized controlled studies were included in this meta-analysis (telehealth: 135,875, control: 94,275). It was seen that the number of ultrasound (p &lt; 0.01) and face-to-face visits (p &lt; 0.01), fasting insulin (p &lt; 0.01), hemoglobin A1C before delivery (p &lt; 0.01), and emergency cesarean section rates (p = 0.05) were lower in the telehealth group. In the telehealth group, the women's use of antenatal corticosteroids (p = 0.03) and hypoglycemic medication at delivery (p = 0.03), the total of nursing interventions (p &lt; 0.01), compliance with actual blood glucose measurements (p &lt; 0.01), induction intervention at delivery (p = 0.003), and maternal mortality (p &lt; 0.001) rates were higher. Two groups were similar in terms of the use of medical therapy, total gestational weight gain, health problems related to pregnancy, mode and complications of delivery, maternal intensive care unit admission, fetal-neonatal growth and development, neonatal health problems and mortality, follow-up, and care costs. Discussion: Telehealth and routine care yielded similar maternal/neonatal health and cost outcomes. It can be said that telehealth is a safe technique to work with in the management of high-risk pregnancies. (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>10.1177/1357633X221087867</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Journal of Telemedicine and Telecare</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Gunes Ozturk</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>sexualfunctionafterchildbirth:ameta-analysisbasedonmodeofdelivery;2023;alimi</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>sexual function after childbirth: a meta-analysis based on mode of delivery</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Alimi, Rasoul;Marvi, Nahid;Azmoude, Elham;Heidarian Miri, Hamid;Zamani, Maryam</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Although many women report sexual dysfunction in the postpartum period, controversial research has been reported the relationship between delivery mode and sexual function. This meta-analysis aimed to investigate the sexual function after childbirth and identify the difference of sexual function based on the female sexual function index (FSFI) questionnaire in women with elective cesarean section, vaginal delivery with episiotomy and vaginal delivery without episiotomy. Studies were found by searching in Medline, PubMed, Web of Science, Scopus and considering the references of the related papers from their start dates until September 2021. All observational studies in English that reported the mean and SD of score of sexual function and its domains based on the mode of delivery were included in this meta-analysis. Random effect model was used to combine the results of included studies on female sexual function and its subdomains. Finally, 17 articles with a total population of 3410 were included in the meta-analysis. Total mean (95 percent CI) of sexual function was 24.27 (22.82, 25.72) with substantial heterogeneity among studies (kh2 = 7487.63, P &lt; .001; I2 = 99.45). In subgroup analyses, the mean score of sexual function was significantly differed in terms of time elapsed since delivery (P = .04) and studied country (P &lt; .001). But, the mode of delivery has no significant effect on postpartum sexual function and subdomains. The result indicated that elective cesarean section, vaginal delivery with episiotomy, vaginal delivery without episiotomy are not associated with the female sexual function. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>10.1080/03630242.2022.2158412</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>36576252</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Women &amp; Health</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Alimi</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>effectsofketamineandesketamineonpreventingpostpartumdepressionaftercesareandelivery:ameta-analysis;2024;li</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>effects of ketamine and esketamine on preventing postpartum depression after cesarean delivery: a meta-analysis</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>2024</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Li, Shuying;Zhou, Wenqin;Li, Ping;Lin, Rongqian</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Background: Ketamine and esketamine has been suggested to have potential efficacy in preventing postpartum depression (PPD) recent years. The aim of this meta-analysis was to evaluate the effectiveness of ketamine and esketamine on PPD after cesarean delivery. Methods: We systematically searched PubMed, Embase, and the Cochrane Library for studies investigating the efficacy of ketamine and esketamine in preventing PPD. The primary outcomes of this study were risk ratios (RRs) and EPDS scores (Edinburgh Postnatal Depression Scale) in relation to PPD after ketamine and esketamine. The second outcomes were the postoperative adverse events. Results: Thirteen randomized controlled trials (RCTs) and one retrospective study including 2916 patients were analyzed, including six on the use of ketamine and eight on the use of esketamine. The risk ratios and EPDS scores of PPD were significantly decreased in the ketamine/esketamine group compared to those in the control group in one week and four weeks postoperative periods. Subgroup analyses showed that high dosage, administrated in patient controlled intravenous analgesia (PCIA) method and only esketamine exhibited a significant reduction in the incidence and EPDS scores of PPD in one week and four week postoperative. However, the incidences of postoperative adverse events, such as dizziness, diplopia, hallucination, and headache were significantly higher in the ketamine/esketamine group than that in the control group. Conclusion: Ketamine and esketamine appear to be effective in preventing PPD in the one week and four week postoperative periods after cesarean delivery with moderate certainty of evidence. But they can also lead to some short-term complications too. Future high-quality studies are needed to confirm the efficacy of ketamine and esketamine in different countries. (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>10.1016/j.jad.2024.01.202</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>38286233</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Journal of Affective Disorders</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Li</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>environmentalfactorsassociatedwithautismspectrumdisorderinsoutherneurope:asystematicreview;2023;kazantzidou</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>environmental factors associated with autism spectrum disorder in southern europe: a systematic review</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Kazantzidou, Panagiota;Antonopoulou, Katerina;Costarelli, Vasiliki;Papanikolaou, George</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>The aetiology of autism spectrum disorder (ASD) is heterogeneous and is attributed to the concurrent interaction of a number of genetic and environmental factors. The steady increase in ASD rates in recent years makes the detection and study of environmental risk factors increasingly important. This systematic review identifies potential environmental factors associated with ASD focusing specifically on recent studies conducted in selected Southern European countries. Nine relevant studies were selected for this systematic review. Results indicate that ASD in Southern Europe is associated with a variety of prenatal, perinatal and postnatal environmental factors, including stressful early life events, maternal infection during pregnancy, delivery mode and perinatal complications or breastfeeding problems in the offspring. Specially designed, large population-based birth cohort studies are needed in Southern Europe, to allow precise assessment of potential environmental confounders and elucidate their association with ASD. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>10.1080/20473869.2023.2215012</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>International Journal of Developmental Disabilities</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Journal;</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Kazantzidou</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>useofswedishsmokelesstobaccoduringpregnancy:asystematicreviewofpregnancyandearlylifehealthrisk;2023;brinchmann</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>use of swedish smokeless tobacco during pregnancy: a systematic review of pregnancy and early life health risk</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Brinchmann, Bendik, C.;Vist, Gunn, E.;Becher, Rune;Grimsrud, Tom, K.;Elvsaas, Ida-Kristin, Orjasaeter;Underland, Vigdis;Holme, Jorn, A.;Carlsen, Karin C., Lodrup;Kreyberg, Ina;Nordhagen, Live, S.;Bains, Karen Eline, Stensby;Carlsen, Kai-Hakon;Alexander, Jan;Valen, Hakon</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Background and Aims: Smokeless tobacco is a heterogeneous product group with diverse composition and prevalence globally. Tobacco use during pregnancy is concerning due to the risk of adverse pregnancy outcomes and effects on child health. Nicotine may mediate several of these effects. This systematic review measured health outcomes from Swedish smokeless tobacco (snus) use during pregnancy. Method: Literature search was conducted by an information specialist in May 2022. We included human studies of snus use during pregnancy compared with no tobacco use, assessed risk of bias, conducted a meta-analysis and assessed confidence in effectestimates using Grading of Recommendations, Assessment, Development and Evaluations (GRADE). Results: We included 18 cohort studies (42 to 1 006 398 participants). Snus use during pregnancy probably (moderate confidence in risk estimates) increase the risk of neonatal apnea, adjusted odds ratio 95% confidence interval [aOR (95% CI)] 1.96 (1.30 to 2.96). Snus use during pregnancy possibly (low confidence in risk estimates) increase the risk of stillbirths aOR 1.43 (1.02 to 1.99), extremely premature births aOR 1.69 (1.17 to 2.45), moderately premature birth aOR 1.26 (1.15 to 1.38), SGA aOR 1.26 (1.09 to 1.46), reduced birth weight mean difference of 72.47 g (110.58 g to 34.35 g reduction) and oral cleft malformations aOR 1.48 (1.00 to 2.21). It is uncertain (low confidence in risk estimates, CI crossing 1) whether snus use during pregnancy affects risk of preeclampsia aOR 1.11 (0.97 to 1.28), antenatal bleeding aOR 1.15 (0.92 to 1.44) and very premature birth aOR 1.26 (0.95 to 1.66). Risk of early neonatal mortality and altered heart rate variability is uncertain, very low confidence. Snus using mothers had increased prevalence of caesarean sections, low confidence. Conclusions: This systematic review reveals that use of smokeless tobacco (snus) during pregnancy may adversely impact the developing child. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>10.1111/add.16114</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>36524899</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Addiction</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Brinchmann</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>riskfactorsofpostpartumdepressionanddepressivesymptoms:umbrellareviewofcurrentevidencefromsystematicreviewsandmeta-analysesofobservationalstudies;2022;gastaldon</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>risk factors of postpartum depression and depressive symptoms: umbrella review of current evidence from systematic reviews and meta-analyses of observational studies</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Gastaldon, Chiara;Solmi, Marco;Correll, Christoph, U.;Barbui, Corrado;Schoretsanitis, Georgios</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Background: Evidence on risk factors for postpartum depression (PPD) are fragmented and inconsistent. Aims To assess the strength and credibility of evidence on risk factors of PPD, ranking them based on the umbrella review methodology. Method: Databases were searched until 1 December 2020, for systematic reviews and meta-analyses of observational studies. Two reviewers assessed quality, credibility of associations according to umbrella review criteria (URC) and evidence certainty according to Grading of Recommendations-Assessment-Development-Evaluations criteria. Results: Including 185 observational studies (n = 3 272 093) from 11 systematic reviews, the association between premenstrual syndrome and PPD was the strongest (highly suggestive: odds ratio 2.20, 95%CI 1.81-2.68), followed by violent experiences (highly suggestive: odds ratio (OR) = 2.07, 95%CI 1.70-2.50) and unintended pregnancy (highly suggestive: OR=1.53, 95%CI 1.35-1.75). Following URC, the association was suggestive for Caesarean section (OR = 1.29, 95%CI 1.17-1.43), gestational diabetes (OR = 1.60, 95%CI 1.25-2.06) and 5-HTTPRL polymorphism (OR = 0.70, 95%CI 0.57-0.86); and weak for preterm delivery (OR = 2.12, 95%CI 1.43-3.14), anaemia during pregnancy (OR = 1.47, 95%CI 1.17-1.84), vitamin D deficiency (OR = 3.67, 95%CI 1.72-7.85) and postpartum anaemia (OR = 1.75, 95%CI 1.18-2.60). No significant associations were found for medically assisted conception and intra-labour epidural analgesia. No association was rated as 'convincing evidence'. According to GRADE, the certainty of the evidence was low for Caesarean section, preterm delivery, 5-HTTLPR polymorphism and anaemia during pregnancy, and 'very low' for remaining factors. Conclusions: The most robust risk factors of PDD were premenstrual syndrome, violent experiences and unintended pregnancy. These results should be integrated in clinical algorithms to assess the risk of PPD. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>10.1192/bjp.2021.222</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>The British Journal of Psychiatry</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Gastaldon</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>postpartumhemorrhageandpostpartumdepression:asystematicreviewandmeta-analysisofobservationalstudies;2023;schoretsanitis</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>postpartum hemorrhage and postpartum depression: a systematic review and meta-analysis of observational studies</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>2023</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Schoretsanitis, Georgios;Gastaldon, Chiara;Ochsenbein-Koelble, Nicole;Olbrich, Sebastian;Barbui, Corrado;Seifritz, Erich</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Objective To assess the postpartum depression (PPD) risk in women with postpartum hemorrhage (PPH) and moderators. Methods We identified observational studies of PPD rates in women with versus without PPH in Embase/Medline/PsychInfo/Cinhail in 09/2022. Study quality was evaluated using the Newcastle-Ottawa-Scale. Our primary outcome was the odds ratio (OR, 95% confidence intervals [95%CI]) of PPD in women with versus without PPH. Meta-regression analyses included the effects of age, body mass index, marital status, education, history of depression/anxiety, preeclampsia, antenatal anemia and C-section; subgroup analyses were based on PPH and PPD assessment methods, samples with versus without history of depression/anxiety, from low-/middle- versus high-income countries. We performed sensitivity analyses after excluding poor-quality studies, cross-sectional studies and sequentially each study. Results One, five and three studies were rated as good-, fair- and poor-quality respectively. In nine studies (k = 10 cohorts, n = 934,432), women with PPH were at increased PPD risk compared to women without PPH (OR = 1.28, 95% CI = 1.13 to 1.44, p &lt; 0.001), with substantial heterogeneity (I2 = 98.9%). Higher PPH-related PPD ORs were estimated in samples with versus without history of depression/anxiety or antidepressant exposure (OR = 1.37, 95%CI = 1.18 to 1.60, k = 6, n = 55,212, versus 1.06, 95%CI = 1.04 to 1.09, k = 3, n = 879,220, p &lt; 0.001) and in cohorts from low-/middle- versus high-income countries (OR = 1.49, 95%CI = 1.37 to 1.61, k = 4, n = 9197, versus 1.13, 95%CI = 1.04 to 1.23, k = 6, n = 925,235, p &lt; 0.001). After excluding low-quality studies the PPD OR dropped (1.14, 95%CI = 1.02 to 1.29, k = 6, n = 929,671, p = 0.02). Conclusions Women with PPH had increased PPD risk amplified by history of depression/anxiety, whereas more data from low-/middle-income countries are required. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>10.1111/acps.13583</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>37286177</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Acta Psychiatrica Scandinavica</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Journal;</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Schoretsanitis</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>polycysticovarysyndromeandpostpartumdepression:asystematicreviewandmeta-analysisofobservationalstudies;2022;schoretsanitis</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>polycystic ovary syndrome and postpartum depression: a systematic review and meta-analysis of observational studies</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Schoretsanitis, Georgios;Gastaldon, Chiara;Kalaitzopoulos, Dimitrios, R.;Ochsenbein-Koelble, Nicole;Barbui, Corrado;Seifritz, Erich</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Objective: To estimate the risk of postpartum depression (PPD) in women with polycystic ovary syndrome (PCOS) and assess related moderators. Methods: Observational studies reporting on PPD rates in women with vs. without PCOS were identified in Embase/Medline/PsychInfo/Cinhail in 03/2021 since data inception. Quality of studies was evaluated using the Newcastle-Ottawa-Scale. The primary outcome was the odds ratio (OR, 95% confidence intervals [95%CI]) of PPD in women with vs. without PCOS. Meta-regression analyses included the effects of age, body mass index, percent smokers, history of depression, preterm delivery, hypertension during pregnancy, gestational diabetes and cesarian section as well as subgroup analyses based on the assessment methods for PCOS and PPD. Sensitivity analyses after excluding poor quality studies and cross-sectional studies and sequentially excluding each study were performed. Results: One study was rated as good, two as fair and three as low-quality. In six studies (n = 934,922), 44,167 women with PCOS were at increased PPD risk compared to 890,755 women without PCOS (OR = 1.45, 95%CI = 1.18 to 1.79, p &lt; 0.001). When excluding one study that underestimated PCOS prevalence, we estimated an OR of 1.59 (95%CI = 1.56 to 1.62, p &lt; 0.001) with reduced heterogeneity (I2 = 45.3%). Higher ORs of PPD in women with PCOS were moderated by lower percentage of preterm delivery (co-efficient -0.07, 95%CI = -0.1 to -0.04, p &lt; 0.001). After excluding low-quality studies yielded an OR of 1.58 (95%CI = 1.56 to 1.59, p &lt; 0.001) with heterogeneity dropping (I2 = 14.0%). Limitations: The methodological heterogeneity of available studies. Conclusions: Women with PCOS are at elevated PPD risk with risk moderators requiring further research. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>10.1016/j.jad.2021.12.044</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Journal of Affective Disorders</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Schoretsanitis</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
-        <is>
-          <t>riskfactorsforsevereperineallacerationsduringchildbirth:asystematicreviewandmeta-analysisofcohortstudies;2022;hu</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>risk factors for severe perineal lacerations during childbirth: a systematic review and meta-analysis of cohort studies</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Hu, Yinchu;Lu, Hong;Huang, Qifang;Ren, Lihua;Wang, Na;Huang, Jing;Yang, Minghui;Cao, Linlin</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Aims and objectives To evaluate and quantify the best available evidence regarding risk factors for severe perineal lacerations. Background Many studies have evaluated the risk factors for severe perineal lacerations. However, the results of those studies are inconsistent, and meta-analysis which thoroughly evaluates the risk factors for severe perineal lacerations is still lacking. Design Systematic review and meta-analysis of cohort studies based on the PRISMA guideline. Methods PubMed, Embase, the Cochrane Library, CINAHL, ClinicalTrials.gov, CNKI, Wanfang Data, VIP and SinoMed were systematically searched for cohort studies reporting at least one risk factor for severe perineal lacerations from 1 January 2000 to 2 June 2021. Two reviewers independently conducted quality appraisal by NOS scale and extracted data. Data synthesis was conducted via RevMan 5.3 using a random-effects or fixed-effects model. Results A total of 47 studies with 7,043,218 women were included. The results showed that prior caesarean delivery (OR: 1.46, 95% CI 1.12-1.92) and pre-pregnant underweight (OR: 1.31, 95% CI 1.22-1.41) significantly increased the risk of severe perineal lacerations. The results also demonstrated that episiotomy was protective against severe perineal lacerations in forceps delivery (OR: 0.56, 95% CI 0.42-0.74), but not spontaneous vaginal delivery (OR: 1.30, 95% CI 0.81-2.07) or vacuum delivery (OR: 0.76, 95% CI 0.45-1.28). Nulliparity, foetus in occipitoposterior or occipitotransverse position, and midline episiotomy were also independent risk factors for severe perineal lacerations. Conclusions Severe perineal lacerations are associated with many factors, and evidence-based risk assessment tools are needed to guide the midwives and obstetricians to estimate women's risk of severe perineal lacerations. Relevance to clinical practice This systematic review and meta-analysis identified some important risk factors for severe perineal lacerations, which provides comprehensive insights to guide the midwives to assess women's risk for severe perineal lacerations and take appropriate preventive measures to decrease the risk. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>10.1111/jocn.16438</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Journal of Clinical Nursing</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Journal;</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Hu</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>theassociationofbirthbycaesareansectionandcognitiveoutcomesinoffspring:asystematicreview;2021;blake</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>the association of birth by caesarean section and cognitive outcomes in offspring: a systematic review</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>2021</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Blake, Julie, A.;Gardner, Madeleine;Najman, Jake;Scott, James, G.</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Purpose: Studies have reported children born by caesarean section are more likely to have lower cognitive outcomes compared to those born by vaginal delivery. This paper reviews the literature examining caesarean birth and offspring cognitive outcomes. Methods: A systematic search for observational studies or case-control studies that compared cognitive outcomes of people born by caesarean section with those born by vaginal delivery was conducted in six databases (Medline, PubMed, EMBASE, PsychInfo, CINAHL, Web of Science) from inception until December 2019 according to the Preferred Reporting Items for Systematic Reviews and Meta-Analyses (PRISMA) guidelines. Studies were assessed for quality and a narrative synthesis was undertaken considering the evidence for a causal relationship according to the Bradford Hill Criteria. Results: A total of seven studies were identified. Of these, four found a significant association between elective and emergency caesarean birth and reduction in offspring cognitive performance as measured by school performance or validated cognitive testing. Three studies found no association. There was variability in the quality of the studies, assessment of the reason for caesarean section (emergency vs elective), measurement of outcomes and adjustment for confounding factors. Conclusion: The evidence of an association between CS birth and lower offspring cognitive functioning is inconsistent. Based on currently available data, there is no evidence that a causal association exists. To better examine this association, future studies should (a) distinguish elective and emergency caesareans, (b) adequately adjust for confounding variables and (c) have valid outcome measures of cognition. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>10.1007/s00127-020-02008-2</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>33388795</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Social Psychiatry and Psychiatric Epidemiology: The International Journal for Research in Social and Genetic Epidemiology and Mental Health Services</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Blake</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
-        <is>
-          <t>riskfactorsforneonatalbrachialplexuspalsy:asystematicreviewandmeta-analysis;2020;vanderlooven</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>risk factors for neonatal brachial plexus palsy: a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>2020</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Van der Looven, Ruth;Le Roy, Laura;Tanghe, Emma;Samijn, Bieke;Roets, Ellen;Pauwels, Nele;Deschepper, Ellen;De Muynck, Martine;Vingerhoets, Guy;Van den Broeck, Christine</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Aim: To provide a comprehensive update on the most prevalent, significant risk factors for neonatal brachial plexus palsy (NBPP). Method: Cochrane CENTRAL, MEDLINE, Web of Science, Embase, and ClinicalTrials.gov were searched for relevant publications up to March 2019. Studies assessing risk factors of NBPP in relation to typically developing comparison individuals were included. Meta-analysis was performed for the five most significant risk factors, on the basis of the PRISMA statement and MOOSE guidelines. Pooled odds ratios (ORs), 95% confidence intervals (CIs), and across-study heterogeneity (I2) were reported. Reporting bias and quality of evidence was rated. In addition, we assessed the incidence of NBPP. Results: Twenty-two observational studies with a total sample size of 29 419 037 live births were selected. Significant risk factors included shoulder dystocia (OR 115.27; 95% CI 81.35-163.35; I2 = 92%), macrosomia (OR 9.75; 95% CI 8.29-11.46; I2 = 70%), (gestational) diabetes (OR 5.33; 95% CI 3.77-7.55; I2 = 59%), instrumental delivery (OR 3.8; 95% CI 2.77-5.23; I2 = 77%), and breech delivery (OR 2.49; 95% CI 1.67-3.7; I2 = 70%). Caesarean section appeared as a protective factor (OR 0.13; 95% CI 0.11-0.16; I2 = 41%). The pooled overall incidence of NBPP was 1.74 per 1000 live births. It has decreased in recent years. Interpretation: The incidence of NBPP is decreasing. Shoulder dystocia, macrosomia, maternal diabetes, instrumental delivery, and breech delivery are risk factors for NBPP. Caesarean section appears as a protective factor. What this paper adds The overall incidence of neonatal brachial plexus palsy is 1.74 per 1000 live births. The incidence has declined significantly. Shoulder dystocia, macrosomia, maternal diabetes, instrumental delivery, and breech delivery are the main risk factors. Prevention is difficult owing to unpredictability and often labour-related risk. (PsycInfo Database Record (c) 2020 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>10.1111/dmcn.14381</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>31670385</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Developmental Medicine &amp; Child Neurology</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Van der Looven</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>prenatal,perinatalandneonatalriskfactorsforperinatalarterialischaemicstroke:asystematicreviewandmeta-analysis;2017;li</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>prenatal, perinatal and neonatal risk factors for perinatal arterial ischaemic stroke: a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>2017</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Li, C.;Miao, J., K.;Xu, Y.;Hua, Y., Y.;Ma, Q.;Zhou, L., L.;Liu, H., J.;Chen, Q., X.</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>The aim of the present study was to perform a meta-analysis of published data to determine the significance of clinical factors and exposures to the risk of perinatal arterial ischaemic stroke (PAIS) and provide guidance for clinical diagnosis and treatment. A comprehensive literature search of the PubMed, Embase, MEDLINE and Cochrane Library databases for relevant observational studies (cohort/case-control) from March 1984 to March 2016 was undertaken. Two review authors independently examined the full text records to determine which studies met the inclusion criteria and evaluated risk factors for PAIS. Risk ratios, odds ratios and 95% confidence intervals were estimated. A total of 11 studies were included in the analyses. Intrapartum fever &gt; 38degC, pre-eclampsia, oligohydramnios, primiparity, forceps delivery, vacuum delivery, fetal heart rate abnormalities, abnormal cardiotocography tracing, cord abnormalities, birth asphyxia, emergency caesarean section, tight nuchal cord, meconium-stained amniotic fluid, umbilical arterial pH &lt; 7.10, Apgar score at 5 min &lt; 7, resuscitation at birth, hypoglycaemia, male gender and small for gestational age were identified as risk factors for PAIS. This systemic review and meta-analysis provides a preliminary evidence-based assessment of the risk factors for PAIS. Patients with any of the risk factors identified in this analysis should be given careful consideration to ensure the prevention of PAIS. Future studies focusing on the combined effects of multiple prenatal, perinatal and neonatal risk factors for PAIS are warranted. (PsycINFO Database Record (c) 2017 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>10.1111/ene.13337</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>28646492</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>European Journal of Neurology</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Li</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>in-uteroandperinatalinfluencesonsuiciderisk:asystematicreviewandmeta-analysis;2019;orri</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>in-utero and perinatal influences on suicide risk: a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>2019</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Orri, Massimiliano;Gunnell, David;Richard-Devantoy, Stephane;Bolanis, Despina;Boruff, Jill;Turecki, Gustavo;Geoffroy, Marie-Claude</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Background: Adverse in-utero and perinatal conditions might contribute to an increased suicide risk throughout the lifespan; however, existing evidence is sparse and contradictory. We aimed to investigate in-utero and perinatal exposures associated with suicide, suicide attempt, and suicidal ideation. Methods: We did a systematic review and meta-analysis and searched MEDLINE, Embase, and PsycINFO from inception to Jan 24, 2019, for population-based prospective studies that investigated the association between in-utero and perinatal factors and suicide, suicide attempt, and suicidal ideation. Only papers published in English in peer-reviewed journals were considered. Two researchers independently extracted formal information (eg, country, year, duration of follow-up) and number of cases and non-cases exposed and non-exposed to each risk factor. We calculated pooled odds ratios (ORs) with 95% CIs using random-effects models and used meta-regression to investigate heterogeneity. This study was registered with PROSPERO, number CRD42018091205. Findings: We identified 42 eligible studies; they had a low risk of bias (median quality score 9/9 [IQR 8-9]). Family or parental characteristics, such as high birth order (eg, for fourth-born or later-born vs first-born, pooled OR 1*51 [95% CIs 1*21-1*88]), teenage mothers (1*80 [1*52-2*14]), single mothers (1*57 [1*31-1*89]); indices of socioeconomic position, such as low maternal (1*36 [1*28-1*46]) and paternal (1*38 [1*27-1*51]) education; and fetal growth (eg, low birthweight 1*30 [1*09-1*55] and small for gestational age 1*18 [1*00-1*40]) were associated with higher suicide risk. Father's age, low gestational age, obstetric characteristics (eg, caesarean section), and condition or exposure during pregnancy (eg, maternal smoking or hypertensive disease) were not associated with higher suicide risk. Similar patterns of associations were observed for suicide attempt and suicidal ideation; however, these results were based on a lower number of studies. In meta-regression, differences in length of follow-up explained most between-study heterogeneity (inital I 2 ranged from 0 to 79*5). Interpretation: These findings suggest that prenatal and perinatal characteristics are associated with increased suicide risk during the life course, supporting the developmental origin of health and diseases hypothesis for suicide. The low number of studies for some risk factors, especially for suicide attempt and ideation, leaves gaps in knowledge that need to be addressed. The mechanisms underlying the reported associations and their causal nature still remain unclear. (PsycINFO Database Record (c) 2019 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>10.1016/S2215-0366(19)30077-X</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>31029623</v>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>The Lancet Psychiatry</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Orri</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>doescaesareansectionaffectbreastfeedingpracticesinchina?asystematicreviewandmeta-analysis;2017;zhao</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>does caesarean section affect breastfeeding practices in china? a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>2017</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Zhao, Jian;Zhao, Yun;Du, Mengran;Binns, Colin, W.;Lee, Andy, H.</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Objectives: To ascertain the association between caesarean delivery and breastfeeding practices in China. Methods: We conducted a systematic review and meta-analysis following the Preferred Reporting Items for Systematic Reviews and Meta-Analyses (PRISMA) and Meta-analysis Of Observational Studies in Epidemiology (MOOSE) guidelines. Electronic databases of CNKI, Medline, EMBASE, CINAHL, ProQuest and Science Direct were searched and screened to identify relevant articles from January 1990 to June 2015. Both fixed and random effect meta-analysis techniques were used to estimate the pooled effect size between caesarean delivery and breastfeeding outcomes at different time points. Sensitivity analysis and publication bias test were also conducted. Results: Forty six studies were eligible for the qualitative synthesis of systematic review; among them, 27 studies were included for the meta-analysis. At the early postpartum period, the odds of exclusive breastfeeding after caesarean section was 47% (pooled OR 0.53, 95% CI 0.41, 0.68) lower than that after vaginal delivery. At 4 months postpartum, the odds of breastfeeding was similarly lower (pooled OR 0.61, 95% CI 0.53, 0.71) for caesarean mothers. Substantial heterogeneity among studies was detected for both breastfeeding outcomes. Subgroup analyses stratified by study design, time points of breastfeeding outcomes and definitions of breastfeeding all confirmed the negative association between caesarean section and breastfeeding prevalence. Conclusions: In China, breastfeeding practices were affected adversely by caesarean delivery. Therefore, health policy to improve breastfeeding outcomes should take this into consideration. (PsycINFO Database Record (c) 2017 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>10.1007/s10995-017-2369-x</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>29019000</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Maternal and Child Health Journal</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Zhao</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>theimpactofnegativechildbirthexperienceonfuturereproductivedecisions:aquantitativesystematicreview;2018;shorey</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>the impact of negative childbirth experience on future reproductive decisions: a quantitative systematic review</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>2018</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Shorey, Shefaly;Yang, Yen, Yen;Ang, Emily</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Aim: The aim of this study was to systematically retrieve, critique and synthesize available evidence regarding the association between negative childbirth experiences and future reproductive decisions. Background: A child's birth is often a joyous event; however, there is a proportion of women who undergo negative childbirth experiences that have long-term implications on their reproductive decisions. Design: A systematic review of quantitative studies was undertaken using Joanna Briggs Institute's methods. Review methods: A search was carried out in CINAHL Plus with Full Text, Embase, PsycINFO, PubMed, Scopus and Web of Science from January 1996-July 2016. Studies that fulfilled the inclusion criteria were assessed by two independent reviewers using the Joanna Briggs Institute's Critical Appraisal Tools. Data were extracted under subheadings adapted from the institute's data extraction forms. Results: Twelve studies, which examined either one or more influences of negative childbirth experiences, were identified. The included studies were either cohort or cross-sectional designs. Five studies observed positive associations between prior negative childbirth experiences and decisions to not have another child, three studies found positive associations between negative childbirth experiences and decisions to delay a subsequent birth and six studies concluded positive associations between negative childbirth experiences and maternal requests for caesarean section in subsequent pregnancies. Conclusion: To receive a holistic understanding on negative childbirth experiences, a suitable definition and validated measuring tools should be used to understand this phenomenon. Future studies or reviews should include a qualitative component and/or the exploration of specific factors such as cultural and regional differences that influence childbirth experiences. (PsycINFO Database Record (c) 2019 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>10.1111/jan.13534</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>29394456</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Journal of Advanced Nursing</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Shorey</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
-        <is>
-          <t>feedingneonatesbycup:asystematicreviewoftheliterature;2016;mckinney</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>feeding neonates by cup: a systematic review of the literature</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>2016</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>McKinney, Christy, M.;Glass, Robin, P.;Coffey, Patricia;Rue, Tessa;Vaughn, Matthew, G.;Cunningham, Michael</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Objective: WHO and UNICEF recommend cup feeding for neonates unable to breastfeed in low-resource settings. In developed countries, cup feeding in lieu of bottle feeding in the neonatal period is hypothesized to improve breastfeeding outcomes for those initially unable to breastfeed. Our aim was to synthesize the entire body of evidence on cup feeding. Methods: We searched domestic and international databases for original research. Our search criteria required original data on cup feeding in neonates published in English between January 1990 and December 2014. Results: We identified 28 original research papers. Ten were randomized clinical trials, 7 non-randomized intervention studies, and 11 observational studies; 11 were conducted in developing country. Outcomes evaluated included physiologic stability, safety, intake, duration, spillage, weight gain, any and exclusive breastfeeding, length of hospital stay, compliance, and acceptability. Cup feeding appears to be safe though intake may be less and spillage greater relative to bottle or tube feeding. Overall, slightly higher proportions of cup fed versus bottle fed infants report any breastfeeding; a greater proportion of cup fed infants reported exclusive breastfeeding at discharge and beyond. Cup feeding increases breastfeeding in subgroups (e.g. those who intend to breastfeed or women who had a Caesarean section). Compliance and acceptability is problematic in certain settings. Conclusions: Further research on long-term breastfeeding outcomes and in low-resource settings would be helpful. Research data on high risk infants (e.g. those with cleft palates) would be informative. Innovative cup feeding approaches to minimize spillage, optimize compliance, and increase breastfeeding feeding are needed. (PsycINFO Database Record (c) 2017 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>10.1007/s10995-016-1961-9</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Maternal and Child Health Journal</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>McKinney</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>birth-relatedperinealtraumainlow-andmiddle-incomecountries:asystematicreviewandmeta-analysis;2019;aguiar</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>birth-related perineal trauma in low- and middle-income countries: a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>2019</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Aguiar, Magda;Farley, Amanda;Hope, Lucy;Amin, Adeela;Shah, Pooja;Manaseki-Holland, Semira</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Introduction: Birth-related perineal trauma (BPT) is a common consequence of vaginal births. When poorly managed, BPT can result in increased morbidity and mortality due to infections, haemorrhage, and incontinence. This review aims to collect data on rates of BPT in low- and middle-income countries (LMICs), through a systematic review and meta-analysis. Methods: The following databases were searched: Medline, Embase, Latin American and Caribbean Health Sciences Literature (LILACs), and the World Health Organization (WHO) regional databases, from 2004 to 2016. Cross-sectional data on the proportion of vaginal births that resulted in episiotomy, second degree tears or obstetric anal sphincter injuries (OASI) were extracted from studies carried out in LMICs by two independent reviewers. Estimates were meta-analysed using a random effects model; results were presented by type of BPT, parity, and mode of birth. Results: Of the 1182 citations reviewed, 74 studies providing data on 334,054 births in 41 countries were included. Five studies reported outcomes of births in the community. In LMICs, the overall rates of BPT were 46% (95% CI 36-55%), 24% (95% CI 17-32%), and 1.4% (95% CI 1.2-1.7%) for episiotomies, second degree tears, and OASI, respectively. Studies were highly heterogeneous with respect to study design and population. The overall reporting quality was inadequate. Discussion: Compared to high-income settings, episiotomy rates are high in LMIC medical facilities. There is an urgent need to improve reporting of BPT in LMICs particularly with regards to births taking in community settings. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>10.1007/s10995-019-02732-5</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>30915627</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Maternal and Child Health Journal</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Aguiar</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
-        <is>
-          <t>epilepsyinpregnancyandreproductiveoutcomes:asystematicreviewandmeta-analysis;2015;viale</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>epilepsy in pregnancy and reproductive outcomes: a systematic review and meta-analysis</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>2015</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Viale, Luz;Allotey, John;Cheong-See, Fiona;Arroyo-Manzano, David;Mccorry, Dougall;Bagary, Manny;Mignini, Luciano;Khan, Khalid, S;Zamora, Javier;Thangaratinam, Shakila</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Background: Antenatal care of women with epilepsy is varied. The association of epilepsy and antiepileptic drug exposure with pregnancy outcomes needs to be quantified to guide management. We did a systematic review and meta-analysis to investigate the association between epilepsy and reproductive outcomes, with or without exposure to antiepileptic drugs. Methods: We searched MEDLINE, Embase, Cochrane, AMED, and CINAHL between Jan 1, 1990, and Jan 21, 2015, with no language or regional restrictions, for observational studies of pregnant women with epilepsy, which assessed the risk of obstetric complications in the antenatal, intrapartum, or postnatal period, and any neonatal complications. We used the Newcastle-Ottawa Scale to assess the methodological quality of the included studies, risk of bias in the selection and comparability of cohorts, and outcome. We assessed the odds of maternal and fetal complications (excluding congenital malformations) by comparing pregnant women with and without epilepsy and undertook subgroup analysis based on antiepileptic drug exposure in women with epilepsy. We summarised the association as odds ratio (OR; 95% CI) using random effects meta-analysis. The PROSPERO ID of this Systematic Review's protocol is CRD42014007547. Findings: Of 7050 citations identified, 38 studies from low-income and high-income countries met our inclusion criteria (39 articles including 2 837 325 pregnancies). Women with epilepsy versus those without (2 809 984 pregnancies) had increased odds of spontaneous miscarriage (OR 1*54, 95% CI 1*02-2*32; I2 = 67%), antepartum haemorrhage (1*49, 1*01-2*20; I2 = 37%), post-partum haemorrhage (1*29, 1*13-1*49; I2 = 41%), hypertensive disorders (1*37, 1*21-1*55; I2 = 23%), induction of labour (1*67, 1*31-2*11; I2 = 64%), caesarean section (1*40, 1*23-1*58; I2 = 66%), any preterm birth (&lt;37 weeks of gestation; 1*16, 1*01-1*34; I2 = 64%), and fetal growth restriction (1*26, 1*20-1*33; I2 = 1%). The odds of early preterm birth, gestational diabetes, fetal death or stillbirth, perinatal death, or admission to neonatal intensive care unit did not differ between women with epilepsy and those without the disorder. Interpretation: A small but significant association of epilepsy, exposure to antiepileptic drugs, and adverse outcomes exists in pregnancy. This increased risk should be taken into account when counselling women with epilepsy. Funding: EBM CONNECT Collaboration. (PsycINFO Database Record (c) 2016 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>10.1016/S0140-6736(15)00045-8</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>26318519</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>The Lancet</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Viale</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>cesareansectionandriskofpostpartumdepression:ameta-analysis;2017;xu</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>cesarean section and risk of postpartum depression: a meta-analysis</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>2017</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Xu, Hui;Ding, Yu;Ma, Yue;Xin, Xueling;Zhang, Dongfeng</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Objective: The association of cesarean section (CS) with the risk of postpartum depression (PPD) remains controversial. Therefore, we conducted a meta-analysis to explore the association between CS and the risk of PPD. Methods: A systematic literature search was performed in PubMed, Web of Science and Embase databases for relevant articles up to November 2016. Pooled odds ratios (ORs) with 95% confidence intervals (CIs) were calculated with fixed-effects model or random-effects model. Results: A total of 28 studies from 27 articles involving 532,630 participants were included in this meta-analysis. The pooled OR of the association between CS and PPD risk was 1.26 (95% CI: 1.16-1.36). In subgroup analyses stratified by study design [cohort studies: (1.25, 95% CI: 1.10-1.41); case-control studies: (1.25, 95% CI: 1.00-1.56); cross-sectional studies: (1.44, 95% CI: 1.14-1.82)] and adjustment status of complications during pregnancy [adjusted for: (1.29, 95% CI: 1.12-1.48); not-adjusted for: (1.24, 95% CI: 1.13-1.36)], the abovementioned associations remained consistent. The pooled ORs of PPD were 1.15 (95% CI: 0.92-1.43) for elective cesarean section (ElCS) and 1.47 (95% CI: 1.33-1.62) for emergency cesarean section (EmCS). Conclusion: This meta-analysis suggests that CS and EmCS increase the risk of PPD. Further evidence is needed to explore the associations between the specific types of CS and the risk of PPD. (PsycInfo Database Record (c) 2020 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>10.1016/j.jpsychores.2017.04.016</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>28606491</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Journal of Psychosomatic Research</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Xu</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>genderandbirthcohortdifferencesinadultattachmentinchinesecollegestudents:ameta-analysis;2017;shu</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>gender and birth cohort differences in adult attachment in chinese college students: a meta-analysis</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>2017</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Shu, Cong;Chen, Xu;Liu, Ying;Zhang, Xing;Hu, Dengyu;Hu, Na;Liu, Xinyi</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Since China adopted its reform and opening-up policy, the state of society has changed dramatically. Correspondingly, Chinese college students' scores of the Experiences in Close Relationships scale are expected to have changed from 2003 to 2015. A cross-temporal meta-analysis found that Chinese college students' scores of the attachment anxiety subscale increased by 0.2 standard deviations in the past 13years. With a turning point in 2009, the scores of the attachment avoidance subscale increased by 0.58 standard deviations from 2003 to 2009 and decreased by 0.57 standard deviations from 2009 to 2015. Five social indicators including divorce rate, C-section rate, household size, Consumer Price Index, and Gini coefficient showed significant correlation with attachment anxiety. The results from a second meta-analysis showed that there was no gender difference or cohort effect in gender difference in Chinese college students' adult attachment scores. Finally, the explanations and implications of these changes and the insignificant gender difference are discussed. (PsycInfo Database Record (c) 2020 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>10.1016/j.paid.2016.10.012</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Personality and Individual Differences</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Shu</t>
         </is>
       </c>
     </row>
@@ -4703,7 +3446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4765,6 +3508,1264 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>first_author_surname</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>prenatalpsychologicaldistressand11bhsd2geneexpressioninhumanplacentassystematicreviewandmetaanalysis2024tartour</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>prenatal psychological distress and 11b-hsd2 gene expression in human placentas: systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Tartour, Angham, Ibrahim;Chivese, Tawanda;Eltayeb, Safa;Elamin, Fatima, M.;Fthenou, Eleni;Seed Ahmed, Mohammed;Babu, Giridhara, Rathnaiah</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Background: The placenta acts as a buffer to regulate the degree of fetal exposure to maternal cortisol through the 11-Beta Hydroxysteroid Dehydrogenase isoenzyme type 2 (11-b HSD2) enzyme. We conducted a systematic review and meta-analysis to assess the effect of prenatal psychological distress (PPD) on placental 11-b HSD2 gene expression and explore the related mechanistic pathways involved in fetal neurodevelopment. Methods: We searched PubMed, Embase, Scopus, APA PsycInfo(r), and ProQuest Dissertations for observational studies assessing the association between PPD and 11-b HSD2 expression in human placentas. Adjusted regression coefficients (b) and corresponding 95% confidence intervals (CIs) were pooled based on three contextual PPD exposure groups: prenatal depression, anxiety symptoms, and perceived stress. Results: Of 3159 retrieved records, sixteen longitudinal studies involving 1869 participants across seven countries were included. Overall, exposure to PPD disorders showed weak negative associations with the placental 11-b HSD2 gene expression as follows: prenatal depression (b -0.01, 95% CI 0.05-0.02, I2=0%), anxiety symptoms (b -0.02, 95% CI 0.06-0.01, I2=0%), and perceived stress (b -0.01 95% CI 0.06-0.04, I2=62.8%). Third-trimester PPD exposure was more frequently associated with lower placental 11-b HSD2 levels. PPD and placental 11-b HSD2 were associated with changes in cortisol reactivity and the development of adverse health outcomes in mothers and children. Female-offspring were more vulnerable to PPD exposures. Conclusion: The study presents evidence of a modest role of prenatal psychological distress in regulating placental 11-b HSD2 gene expression. Future prospective cohorts utilizing larger sample sizes or advanced statistical methods to enhance the detection of small effect sizes should be planned. Additionally, controlling for key predictors such as the mother's ethnicity, trimester of PPD exposure, mode of delivery, and infant sex is crucial for valid exploration of PPD effects on fetal programming. (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10.1016/j.psyneuen.2024.107060</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Psychoneuroendocrinology</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Tartour</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>maternaloutcomesusingdelayedpushingversusimmediatepushinginthesecondstageoflabouranumbrellareview2024deusalopez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>maternal outcomes using delayed pushing versus immediate pushing in the second stage of labour: an umbrella review</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Deusa-Lopez, Paula;Cuenca-Martinez, Ferran;Sanchez-Martinez, Vanessa;Sempere-Rubio, Nuria</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Introduction: Different systematic reviews have been developed in the last decades about maternal risks of immediate pushing and delayed pushing, depending on the duration of the second stage of labour, but they do not provide conclusive evidence. Aim: The main aim of this overview of systematic reviews was to assess the maternal outcomes using delayed pushing and immediate pushing in the second stage of labour in women receiving epidural analgesia. Methods: We searched systematically in PubMed (Medline), EMBASE, CINAHL, and Scopus (October 26th, 2023). Methodological quality was analysed using AMSTAR and ROBIS scales, and the strength of evidence was established according to the guidelines advisory committee grading criteria. The outcome measures were the duration of the second stage of labour, duration of active pushing, caesarean section, instrumental vaginal birth, spontaneous vaginal birth, fatigue score, perineal lacerations, postpartum haemorrhage, and rate of episiotomy. Seven systematic reviews with and without meta-analysis were included. Results: Results showed that delayed pushing increases the total time of the second stage of labour, although delayed pushing decreases the duration of active pushing with moderate quality of evidence. Mixed results were found with respect to the variables instrumental vaginal birth, spontaneous vaginal birth, and fatigue score although the results favour delayed pushing or show no statistically significant differences with respect to immediate pushing. No favourable results were ever found for immediate pushing with respect to delayed pushing, with a limited quality of evidence. Even so, delayed pushing seems to be associated with a significant increase in spontaneous vaginal birth rates. The results found no significant differences between the immediate pushing and delayed pushing groups in the caesarean section rates, perineal lacerations, postpartum haemorrhage, and episiotomy ratio, with a limited quality of evidence. Conclusions: This study shows that delayed pushing during the second stage of labour produces at least the same maternal outcomes as immediate pushing, although we note that delayed pushing produces an increase of the duration of the second stage of labour, a shorter duration of the active pushing and a tendency to increase spontaneous vaginal birth and to reduce the instrumental vaginal birth rates and fatigue scores. This should be considered clinically. This review was registered in the International Prospective Register of Systematic Reviews PROSPERO (CRD42023397616). (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10.1016/j.ijnurstu.2024.104693</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>International Journal of Nursing Studies</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Deusa-Lopez</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>theimpactoftelehealthapplicationsonpregnancyoutcomesandcostsinhighriskpregnancyasystematicreviewandmetaanalysis2024gunesozturk</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>the impact of telehealth applications on pregnancy outcomes and costs in high-risk pregnancy: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Gunes Ozturk, Gizem;Akyildiz, Deniz;Karacam, Zekiye</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Introduction: Telehealth is an applicable, acceptable, cost-effective, easily accessible, and speedy method for pregnant women. This study aimed to examine the impact of telehealth applications on pregnancy outcomes and costs in highrisk pregnancies. Methods: Studies were selected from PubMed, Science Direct, Web of Science, EBSCO, Scopus, and Clinical Key databases according to the inclusion and exclusion criteria from January to February 2021. Cochrane risk-of-bias tools were used in the quality assessment of the studies. Results: Four observational and eight randomized controlled studies were included in this meta-analysis (telehealth: 135,875, control: 94,275). It was seen that the number of ultrasound (p &lt; 0.01) and face-to-face visits (p &lt; 0.01), fasting insulin (p &lt; 0.01), hemoglobin A1C before delivery (p &lt; 0.01), and emergency cesarean section rates (p = 0.05) were lower in the telehealth group. In the telehealth group, the women's use of antenatal corticosteroids (p = 0.03) and hypoglycemic medication at delivery (p = 0.03), the total of nursing interventions (p &lt; 0.01), compliance with actual blood glucose measurements (p &lt; 0.01), induction intervention at delivery (p = 0.003), and maternal mortality (p &lt; 0.001) rates were higher. Two groups were similar in terms of the use of medical therapy, total gestational weight gain, health problems related to pregnancy, mode and complications of delivery, maternal intensive care unit admission, fetal-neonatal growth and development, neonatal health problems and mortality, follow-up, and care costs. Discussion: Telehealth and routine care yielded similar maternal/neonatal health and cost outcomes. It can be said that telehealth is a safe technique to work with in the management of high-risk pregnancies. (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10.1177/1357633X221087867</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Journal of Telemedicine and Telecare</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Gunes Ozturk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>sexualfunctionafterchildbirthametaanalysisbasedonmodeofdelivery2023alimi</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sexual function after childbirth: a meta-analysis based on mode of delivery</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Alimi, Rasoul;Marvi, Nahid;Azmoude, Elham;Heidarian Miri, Hamid;Zamani, Maryam</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Although many women report sexual dysfunction in the postpartum period, controversial research has been reported the relationship between delivery mode and sexual function. This meta-analysis aimed to investigate the sexual function after childbirth and identify the difference of sexual function based on the female sexual function index (FSFI) questionnaire in women with elective cesarean section, vaginal delivery with episiotomy and vaginal delivery without episiotomy. Studies were found by searching in Medline, PubMed, Web of Science, Scopus and considering the references of the related papers from their start dates until September 2021. All observational studies in English that reported the mean and SD of score of sexual function and its domains based on the mode of delivery were included in this meta-analysis. Random effect model was used to combine the results of included studies on female sexual function and its subdomains. Finally, 17 articles with a total population of 3410 were included in the meta-analysis. Total mean (95 percent CI) of sexual function was 24.27 (22.82, 25.72) with substantial heterogeneity among studies (kh2 = 7487.63, P &lt; .001; I2 = 99.45). In subgroup analyses, the mean score of sexual function was significantly differed in terms of time elapsed since delivery (P = .04) and studied country (P &lt; .001). But, the mode of delivery has no significant effect on postpartum sexual function and subdomains. The result indicated that elective cesarean section, vaginal delivery with episiotomy, vaginal delivery without episiotomy are not associated with the female sexual function. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>10.1080/03630242.2022.2158412</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>36576252</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Women &amp; Health</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Alimi</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>effectsofketamineandesketamineonpreventingpostpartumdepressionaftercesareandeliveryametaanalysis2024li</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>effects of ketamine and esketamine on preventing postpartum depression after cesarean delivery: a meta-analysis</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Li, Shuying;Zhou, Wenqin;Li, Ping;Lin, Rongqian</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Background: Ketamine and esketamine has been suggested to have potential efficacy in preventing postpartum depression (PPD) recent years. The aim of this meta-analysis was to evaluate the effectiveness of ketamine and esketamine on PPD after cesarean delivery. Methods: We systematically searched PubMed, Embase, and the Cochrane Library for studies investigating the efficacy of ketamine and esketamine in preventing PPD. The primary outcomes of this study were risk ratios (RRs) and EPDS scores (Edinburgh Postnatal Depression Scale) in relation to PPD after ketamine and esketamine. The second outcomes were the postoperative adverse events. Results: Thirteen randomized controlled trials (RCTs) and one retrospective study including 2916 patients were analyzed, including six on the use of ketamine and eight on the use of esketamine. The risk ratios and EPDS scores of PPD were significantly decreased in the ketamine/esketamine group compared to those in the control group in one week and four weeks postoperative periods. Subgroup analyses showed that high dosage, administrated in patient controlled intravenous analgesia (PCIA) method and only esketamine exhibited a significant reduction in the incidence and EPDS scores of PPD in one week and four week postoperative. However, the incidences of postoperative adverse events, such as dizziness, diplopia, hallucination, and headache were significantly higher in the ketamine/esketamine group than that in the control group. Conclusion: Ketamine and esketamine appear to be effective in preventing PPD in the one week and four week postoperative periods after cesarean delivery with moderate certainty of evidence. But they can also lead to some short-term complications too. Future high-quality studies are needed to confirm the efficacy of ketamine and esketamine in different countries. (PsycInfo Database Record (c) 2024 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10.1016/j.jad.2024.01.202</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>38286233</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Journal of Affective Disorders</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Li</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>environmentalfactorsassociatedwithautismspectrumdisorderinsoutherneuropeasystematicreview2023kazantzidou</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>environmental factors associated with autism spectrum disorder in southern europe: a systematic review</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Kazantzidou, Panagiota;Antonopoulou, Katerina;Costarelli, Vasiliki;Papanikolaou, George</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>The aetiology of autism spectrum disorder (ASD) is heterogeneous and is attributed to the concurrent interaction of a number of genetic and environmental factors. The steady increase in ASD rates in recent years makes the detection and study of environmental risk factors increasingly important. This systematic review identifies potential environmental factors associated with ASD focusing specifically on recent studies conducted in selected Southern European countries. Nine relevant studies were selected for this systematic review. Results indicate that ASD in Southern Europe is associated with a variety of prenatal, perinatal and postnatal environmental factors, including stressful early life events, maternal infection during pregnancy, delivery mode and perinatal complications or breastfeeding problems in the offspring. Specially designed, large population-based birth cohort studies are needed in Southern Europe, to allow precise assessment of potential environmental confounders and elucidate their association with ASD. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>10.1080/20473869.2023.2215012</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>International Journal of Developmental Disabilities</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Journal;</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Kazantzidou</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>useofswedishsmokelesstobaccoduringpregnancyasystematicreviewofpregnancyandearlylifehealthrisk2023brinchmann</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>use of swedish smokeless tobacco during pregnancy: a systematic review of pregnancy and early life health risk</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Brinchmann, Bendik, C.;Vist, Gunn, E.;Becher, Rune;Grimsrud, Tom, K.;Elvsaas, Ida-Kristin, Orjasaeter;Underland, Vigdis;Holme, Jorn, A.;Carlsen, Karin C., Lodrup;Kreyberg, Ina;Nordhagen, Live, S.;Bains, Karen Eline, Stensby;Carlsen, Kai-Hakon;Alexander, Jan;Valen, Hakon</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Background and Aims: Smokeless tobacco is a heterogeneous product group with diverse composition and prevalence globally. Tobacco use during pregnancy is concerning due to the risk of adverse pregnancy outcomes and effects on child health. Nicotine may mediate several of these effects. This systematic review measured health outcomes from Swedish smokeless tobacco (snus) use during pregnancy. Method: Literature search was conducted by an information specialist in May 2022. We included human studies of snus use during pregnancy compared with no tobacco use, assessed risk of bias, conducted a meta-analysis and assessed confidence in effectestimates using Grading of Recommendations, Assessment, Development and Evaluations (GRADE). Results: We included 18 cohort studies (42 to 1 006 398 participants). Snus use during pregnancy probably (moderate confidence in risk estimates) increase the risk of neonatal apnea, adjusted odds ratio 95% confidence interval [aOR (95% CI)] 1.96 (1.30 to 2.96). Snus use during pregnancy possibly (low confidence in risk estimates) increase the risk of stillbirths aOR 1.43 (1.02 to 1.99), extremely premature births aOR 1.69 (1.17 to 2.45), moderately premature birth aOR 1.26 (1.15 to 1.38), SGA aOR 1.26 (1.09 to 1.46), reduced birth weight mean difference of 72.47 g (110.58 g to 34.35 g reduction) and oral cleft malformations aOR 1.48 (1.00 to 2.21). It is uncertain (low confidence in risk estimates, CI crossing 1) whether snus use during pregnancy affects risk of preeclampsia aOR 1.11 (0.97 to 1.28), antenatal bleeding aOR 1.15 (0.92 to 1.44) and very premature birth aOR 1.26 (0.95 to 1.66). Risk of early neonatal mortality and altered heart rate variability is uncertain, very low confidence. Snus using mothers had increased prevalence of caesarean sections, low confidence. Conclusions: This systematic review reveals that use of smokeless tobacco (snus) during pregnancy may adversely impact the developing child. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>10.1111/add.16114</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>36524899</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Addiction</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Brinchmann</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>riskfactorsofpostpartumdepressionanddepressivesymptomsumbrellareviewofcurrentevidencefromsystematicreviewsandmetaanalysesofobservationalstudies2022gastaldon</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>risk factors of postpartum depression and depressive symptoms: umbrella review of current evidence from systematic reviews and meta-analyses of observational studies</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Gastaldon, Chiara;Solmi, Marco;Correll, Christoph, U.;Barbui, Corrado;Schoretsanitis, Georgios</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Background: Evidence on risk factors for postpartum depression (PPD) are fragmented and inconsistent. Aims To assess the strength and credibility of evidence on risk factors of PPD, ranking them based on the umbrella review methodology. Method: Databases were searched until 1 December 2020, for systematic reviews and meta-analyses of observational studies. Two reviewers assessed quality, credibility of associations according to umbrella review criteria (URC) and evidence certainty according to Grading of Recommendations-Assessment-Development-Evaluations criteria. Results: Including 185 observational studies (n = 3 272 093) from 11 systematic reviews, the association between premenstrual syndrome and PPD was the strongest (highly suggestive: odds ratio 2.20, 95%CI 1.81-2.68), followed by violent experiences (highly suggestive: odds ratio (OR) = 2.07, 95%CI 1.70-2.50) and unintended pregnancy (highly suggestive: OR=1.53, 95%CI 1.35-1.75). Following URC, the association was suggestive for Caesarean section (OR = 1.29, 95%CI 1.17-1.43), gestational diabetes (OR = 1.60, 95%CI 1.25-2.06) and 5-HTTPRL polymorphism (OR = 0.70, 95%CI 0.57-0.86); and weak for preterm delivery (OR = 2.12, 95%CI 1.43-3.14), anaemia during pregnancy (OR = 1.47, 95%CI 1.17-1.84), vitamin D deficiency (OR = 3.67, 95%CI 1.72-7.85) and postpartum anaemia (OR = 1.75, 95%CI 1.18-2.60). No significant associations were found for medically assisted conception and intra-labour epidural analgesia. No association was rated as 'convincing evidence'. According to GRADE, the certainty of the evidence was low for Caesarean section, preterm delivery, 5-HTTLPR polymorphism and anaemia during pregnancy, and 'very low' for remaining factors. Conclusions: The most robust risk factors of PDD were premenstrual syndrome, violent experiences and unintended pregnancy. These results should be integrated in clinical algorithms to assess the risk of PPD. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>10.1192/bjp.2021.222</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>The British Journal of Psychiatry</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Gastaldon</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>postpartumhemorrhageandpostpartumdepressionasystematicreviewandmetaanalysisofobservationalstudies2023schoretsanitis</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>postpartum hemorrhage and postpartum depression: a systematic review and meta-analysis of observational studies</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Schoretsanitis, Georgios;Gastaldon, Chiara;Ochsenbein-Koelble, Nicole;Olbrich, Sebastian;Barbui, Corrado;Seifritz, Erich</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Objective To assess the postpartum depression (PPD) risk in women with postpartum hemorrhage (PPH) and moderators. Methods We identified observational studies of PPD rates in women with versus without PPH in Embase/Medline/PsychInfo/Cinhail in 09/2022. Study quality was evaluated using the Newcastle-Ottawa-Scale. Our primary outcome was the odds ratio (OR, 95% confidence intervals [95%CI]) of PPD in women with versus without PPH. Meta-regression analyses included the effects of age, body mass index, marital status, education, history of depression/anxiety, preeclampsia, antenatal anemia and C-section; subgroup analyses were based on PPH and PPD assessment methods, samples with versus without history of depression/anxiety, from low-/middle- versus high-income countries. We performed sensitivity analyses after excluding poor-quality studies, cross-sectional studies and sequentially each study. Results One, five and three studies were rated as good-, fair- and poor-quality respectively. In nine studies (k = 10 cohorts, n = 934,432), women with PPH were at increased PPD risk compared to women without PPH (OR = 1.28, 95% CI = 1.13 to 1.44, p &lt; 0.001), with substantial heterogeneity (I2 = 98.9%). Higher PPH-related PPD ORs were estimated in samples with versus without history of depression/anxiety or antidepressant exposure (OR = 1.37, 95%CI = 1.18 to 1.60, k = 6, n = 55,212, versus 1.06, 95%CI = 1.04 to 1.09, k = 3, n = 879,220, p &lt; 0.001) and in cohorts from low-/middle- versus high-income countries (OR = 1.49, 95%CI = 1.37 to 1.61, k = 4, n = 9197, versus 1.13, 95%CI = 1.04 to 1.23, k = 6, n = 925,235, p &lt; 0.001). After excluding low-quality studies the PPD OR dropped (1.14, 95%CI = 1.02 to 1.29, k = 6, n = 929,671, p = 0.02). Conclusions Women with PPH had increased PPD risk amplified by history of depression/anxiety, whereas more data from low-/middle-income countries are required. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>10.1111/acps.13583</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>37286177</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Acta Psychiatrica Scandinavica</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Journal;</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Schoretsanitis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>polycysticovarysyndromeandpostpartumdepressionasystematicreviewandmetaanalysisofobservationalstudies2022schoretsanitis</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>polycystic ovary syndrome and postpartum depression: a systematic review and meta-analysis of observational studies</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Schoretsanitis, Georgios;Gastaldon, Chiara;Kalaitzopoulos, Dimitrios, R.;Ochsenbein-Koelble, Nicole;Barbui, Corrado;Seifritz, Erich</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Objective: To estimate the risk of postpartum depression (PPD) in women with polycystic ovary syndrome (PCOS) and assess related moderators. Methods: Observational studies reporting on PPD rates in women with vs. without PCOS were identified in Embase/Medline/PsychInfo/Cinhail in 03/2021 since data inception. Quality of studies was evaluated using the Newcastle-Ottawa-Scale. The primary outcome was the odds ratio (OR, 95% confidence intervals [95%CI]) of PPD in women with vs. without PCOS. Meta-regression analyses included the effects of age, body mass index, percent smokers, history of depression, preterm delivery, hypertension during pregnancy, gestational diabetes and cesarian section as well as subgroup analyses based on the assessment methods for PCOS and PPD. Sensitivity analyses after excluding poor quality studies and cross-sectional studies and sequentially excluding each study were performed. Results: One study was rated as good, two as fair and three as low-quality. In six studies (n = 934,922), 44,167 women with PCOS were at increased PPD risk compared to 890,755 women without PCOS (OR = 1.45, 95%CI = 1.18 to 1.79, p &lt; 0.001). When excluding one study that underestimated PCOS prevalence, we estimated an OR of 1.59 (95%CI = 1.56 to 1.62, p &lt; 0.001) with reduced heterogeneity (I2 = 45.3%). Higher ORs of PPD in women with PCOS were moderated by lower percentage of preterm delivery (co-efficient -0.07, 95%CI = -0.1 to -0.04, p &lt; 0.001). After excluding low-quality studies yielded an OR of 1.58 (95%CI = 1.56 to 1.59, p &lt; 0.001) with heterogeneity dropping (I2 = 14.0%). Limitations: The methodological heterogeneity of available studies. Conclusions: Women with PCOS are at elevated PPD risk with risk moderators requiring further research. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>10.1016/j.jad.2021.12.044</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Journal of Affective Disorders</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Schoretsanitis</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>riskfactorsforsevereperineallacerationsduringchildbirthasystematicreviewandmetaanalysisofcohortstudies2022hu</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>risk factors for severe perineal lacerations during childbirth: a systematic review and meta-analysis of cohort studies</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Hu, Yinchu;Lu, Hong;Huang, Qifang;Ren, Lihua;Wang, Na;Huang, Jing;Yang, Minghui;Cao, Linlin</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Aims and objectives To evaluate and quantify the best available evidence regarding risk factors for severe perineal lacerations. Background Many studies have evaluated the risk factors for severe perineal lacerations. However, the results of those studies are inconsistent, and meta-analysis which thoroughly evaluates the risk factors for severe perineal lacerations is still lacking. Design Systematic review and meta-analysis of cohort studies based on the PRISMA guideline. Methods PubMed, Embase, the Cochrane Library, CINAHL, ClinicalTrials.gov, CNKI, Wanfang Data, VIP and SinoMed were systematically searched for cohort studies reporting at least one risk factor for severe perineal lacerations from 1 January 2000 to 2 June 2021. Two reviewers independently conducted quality appraisal by NOS scale and extracted data. Data synthesis was conducted via RevMan 5.3 using a random-effects or fixed-effects model. Results A total of 47 studies with 7,043,218 women were included. The results showed that prior caesarean delivery (OR: 1.46, 95% CI 1.12-1.92) and pre-pregnant underweight (OR: 1.31, 95% CI 1.22-1.41) significantly increased the risk of severe perineal lacerations. The results also demonstrated that episiotomy was protective against severe perineal lacerations in forceps delivery (OR: 0.56, 95% CI 0.42-0.74), but not spontaneous vaginal delivery (OR: 1.30, 95% CI 0.81-2.07) or vacuum delivery (OR: 0.76, 95% CI 0.45-1.28). Nulliparity, foetus in occipitoposterior or occipitotransverse position, and midline episiotomy were also independent risk factors for severe perineal lacerations. Conclusions Severe perineal lacerations are associated with many factors, and evidence-based risk assessment tools are needed to guide the midwives and obstetricians to estimate women's risk of severe perineal lacerations. Relevance to clinical practice This systematic review and meta-analysis identified some important risk factors for severe perineal lacerations, which provides comprehensive insights to guide the midwives to assess women's risk for severe perineal lacerations and take appropriate preventive measures to decrease the risk. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>10.1111/jocn.16438</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Journal of Clinical Nursing</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Journal;</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Hu</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>theassociationofbirthbycaesareansectionandcognitiveoutcomesinoffspringasystematicreview2021blake</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>the association of birth by caesarean section and cognitive outcomes in offspring: a systematic review</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Blake, Julie, A.;Gardner, Madeleine;Najman, Jake;Scott, James, G.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Purpose: Studies have reported children born by caesarean section are more likely to have lower cognitive outcomes compared to those born by vaginal delivery. This paper reviews the literature examining caesarean birth and offspring cognitive outcomes. Methods: A systematic search for observational studies or case-control studies that compared cognitive outcomes of people born by caesarean section with those born by vaginal delivery was conducted in six databases (Medline, PubMed, EMBASE, PsychInfo, CINAHL, Web of Science) from inception until December 2019 according to the Preferred Reporting Items for Systematic Reviews and Meta-Analyses (PRISMA) guidelines. Studies were assessed for quality and a narrative synthesis was undertaken considering the evidence for a causal relationship according to the Bradford Hill Criteria. Results: A total of seven studies were identified. Of these, four found a significant association between elective and emergency caesarean birth and reduction in offspring cognitive performance as measured by school performance or validated cognitive testing. Three studies found no association. There was variability in the quality of the studies, assessment of the reason for caesarean section (emergency vs elective), measurement of outcomes and adjustment for confounding factors. Conclusion: The evidence of an association between CS birth and lower offspring cognitive functioning is inconsistent. Based on currently available data, there is no evidence that a causal association exists. To better examine this association, future studies should (a) distinguish elective and emergency caesareans, (b) adequately adjust for confounding variables and (c) have valid outcome measures of cognition. (PsycInfo Database Record (c) 2023 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>10.1007/s00127-020-02008-2</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>33388795</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Social Psychiatry and Psychiatric Epidemiology: The International Journal for Research in Social and Genetic Epidemiology and Mental Health Services</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Blake</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>riskfactorsforneonatalbrachialplexuspalsyasystematicreviewandmetaanalysis2020vanderlooven</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>risk factors for neonatal brachial plexus palsy: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Van der Looven, Ruth;Le Roy, Laura;Tanghe, Emma;Samijn, Bieke;Roets, Ellen;Pauwels, Nele;Deschepper, Ellen;De Muynck, Martine;Vingerhoets, Guy;Van den Broeck, Christine</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Aim: To provide a comprehensive update on the most prevalent, significant risk factors for neonatal brachial plexus palsy (NBPP). Method: Cochrane CENTRAL, MEDLINE, Web of Science, Embase, and ClinicalTrials.gov were searched for relevant publications up to March 2019. Studies assessing risk factors of NBPP in relation to typically developing comparison individuals were included. Meta-analysis was performed for the five most significant risk factors, on the basis of the PRISMA statement and MOOSE guidelines. Pooled odds ratios (ORs), 95% confidence intervals (CIs), and across-study heterogeneity (I2) were reported. Reporting bias and quality of evidence was rated. In addition, we assessed the incidence of NBPP. Results: Twenty-two observational studies with a total sample size of 29 419 037 live births were selected. Significant risk factors included shoulder dystocia (OR 115.27; 95% CI 81.35-163.35; I2 = 92%), macrosomia (OR 9.75; 95% CI 8.29-11.46; I2 = 70%), (gestational) diabetes (OR 5.33; 95% CI 3.77-7.55; I2 = 59%), instrumental delivery (OR 3.8; 95% CI 2.77-5.23; I2 = 77%), and breech delivery (OR 2.49; 95% CI 1.67-3.7; I2 = 70%). Caesarean section appeared as a protective factor (OR 0.13; 95% CI 0.11-0.16; I2 = 41%). The pooled overall incidence of NBPP was 1.74 per 1000 live births. It has decreased in recent years. Interpretation: The incidence of NBPP is decreasing. Shoulder dystocia, macrosomia, maternal diabetes, instrumental delivery, and breech delivery are risk factors for NBPP. Caesarean section appears as a protective factor. What this paper adds The overall incidence of neonatal brachial plexus palsy is 1.74 per 1000 live births. The incidence has declined significantly. Shoulder dystocia, macrosomia, maternal diabetes, instrumental delivery, and breech delivery are the main risk factors. Prevention is difficult owing to unpredictability and often labour-related risk. (PsycInfo Database Record (c) 2020 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>10.1111/dmcn.14381</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>31670385</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Developmental Medicine &amp; Child Neurology</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Van der Looven</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>prenatalperinatalandneonatalriskfactorsforperinatalarterialischaemicstrokeasystematicreviewandmetaanalysis2017li</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>prenatal, perinatal and neonatal risk factors for perinatal arterial ischaemic stroke: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Li, C.;Miao, J., K.;Xu, Y.;Hua, Y., Y.;Ma, Q.;Zhou, L., L.;Liu, H., J.;Chen, Q., X.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>The aim of the present study was to perform a meta-analysis of published data to determine the significance of clinical factors and exposures to the risk of perinatal arterial ischaemic stroke (PAIS) and provide guidance for clinical diagnosis and treatment. A comprehensive literature search of the PubMed, Embase, MEDLINE and Cochrane Library databases for relevant observational studies (cohort/case-control) from March 1984 to March 2016 was undertaken. Two review authors independently examined the full text records to determine which studies met the inclusion criteria and evaluated risk factors for PAIS. Risk ratios, odds ratios and 95% confidence intervals were estimated. A total of 11 studies were included in the analyses. Intrapartum fever &gt; 38degC, pre-eclampsia, oligohydramnios, primiparity, forceps delivery, vacuum delivery, fetal heart rate abnormalities, abnormal cardiotocography tracing, cord abnormalities, birth asphyxia, emergency caesarean section, tight nuchal cord, meconium-stained amniotic fluid, umbilical arterial pH &lt; 7.10, Apgar score at 5 min &lt; 7, resuscitation at birth, hypoglycaemia, male gender and small for gestational age were identified as risk factors for PAIS. This systemic review and meta-analysis provides a preliminary evidence-based assessment of the risk factors for PAIS. Patients with any of the risk factors identified in this analysis should be given careful consideration to ensure the prevention of PAIS. Future studies focusing on the combined effects of multiple prenatal, perinatal and neonatal risk factors for PAIS are warranted. (PsycINFO Database Record (c) 2017 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>10.1111/ene.13337</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>28646492</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>European Journal of Neurology</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Li</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>inuteroandperinatalinfluencesonsuicideriskasystematicreviewandmetaanalysis2019orri</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>in-utero and perinatal influences on suicide risk: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Orri, Massimiliano;Gunnell, David;Richard-Devantoy, Stephane;Bolanis, Despina;Boruff, Jill;Turecki, Gustavo;Geoffroy, Marie-Claude</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Background: Adverse in-utero and perinatal conditions might contribute to an increased suicide risk throughout the lifespan; however, existing evidence is sparse and contradictory. We aimed to investigate in-utero and perinatal exposures associated with suicide, suicide attempt, and suicidal ideation. Methods: We did a systematic review and meta-analysis and searched MEDLINE, Embase, and PsycINFO from inception to Jan 24, 2019, for population-based prospective studies that investigated the association between in-utero and perinatal factors and suicide, suicide attempt, and suicidal ideation. Only papers published in English in peer-reviewed journals were considered. Two researchers independently extracted formal information (eg, country, year, duration of follow-up) and number of cases and non-cases exposed and non-exposed to each risk factor. We calculated pooled odds ratios (ORs) with 95% CIs using random-effects models and used meta-regression to investigate heterogeneity. This study was registered with PROSPERO, number CRD42018091205. Findings: We identified 42 eligible studies; they had a low risk of bias (median quality score 9/9 [IQR 8-9]). Family or parental characteristics, such as high birth order (eg, for fourth-born or later-born vs first-born, pooled OR 1*51 [95% CIs 1*21-1*88]), teenage mothers (1*80 [1*52-2*14]), single mothers (1*57 [1*31-1*89]); indices of socioeconomic position, such as low maternal (1*36 [1*28-1*46]) and paternal (1*38 [1*27-1*51]) education; and fetal growth (eg, low birthweight 1*30 [1*09-1*55] and small for gestational age 1*18 [1*00-1*40]) were associated with higher suicide risk. Father's age, low gestational age, obstetric characteristics (eg, caesarean section), and condition or exposure during pregnancy (eg, maternal smoking or hypertensive disease) were not associated with higher suicide risk. Similar patterns of associations were observed for suicide attempt and suicidal ideation; however, these results were based on a lower number of studies. In meta-regression, differences in length of follow-up explained most between-study heterogeneity (inital I 2 ranged from 0 to 79*5). Interpretation: These findings suggest that prenatal and perinatal characteristics are associated with increased suicide risk during the life course, supporting the developmental origin of health and diseases hypothesis for suicide. The low number of studies for some risk factors, especially for suicide attempt and ideation, leaves gaps in knowledge that need to be addressed. The mechanisms underlying the reported associations and their causal nature still remain unclear. (PsycINFO Database Record (c) 2019 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>10.1016/S2215-0366(19)30077-X</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>31029623</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>The Lancet Psychiatry</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Orri</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>doescaesareansectionaffectbreastfeedingpracticesinchinaasystematicreviewandmetaanalysis2017zhao</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>does caesarean section affect breastfeeding practices in china? a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Zhao, Jian;Zhao, Yun;Du, Mengran;Binns, Colin, W.;Lee, Andy, H.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Objectives: To ascertain the association between caesarean delivery and breastfeeding practices in China. Methods: We conducted a systematic review and meta-analysis following the Preferred Reporting Items for Systematic Reviews and Meta-Analyses (PRISMA) and Meta-analysis Of Observational Studies in Epidemiology (MOOSE) guidelines. Electronic databases of CNKI, Medline, EMBASE, CINAHL, ProQuest and Science Direct were searched and screened to identify relevant articles from January 1990 to June 2015. Both fixed and random effect meta-analysis techniques were used to estimate the pooled effect size between caesarean delivery and breastfeeding outcomes at different time points. Sensitivity analysis and publication bias test were also conducted. Results: Forty six studies were eligible for the qualitative synthesis of systematic review; among them, 27 studies were included for the meta-analysis. At the early postpartum period, the odds of exclusive breastfeeding after caesarean section was 47% (pooled OR 0.53, 95% CI 0.41, 0.68) lower than that after vaginal delivery. At 4 months postpartum, the odds of breastfeeding was similarly lower (pooled OR 0.61, 95% CI 0.53, 0.71) for caesarean mothers. Substantial heterogeneity among studies was detected for both breastfeeding outcomes. Subgroup analyses stratified by study design, time points of breastfeeding outcomes and definitions of breastfeeding all confirmed the negative association between caesarean section and breastfeeding prevalence. Conclusions: In China, breastfeeding practices were affected adversely by caesarean delivery. Therefore, health policy to improve breastfeeding outcomes should take this into consideration. (PsycINFO Database Record (c) 2017 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>10.1007/s10995-017-2369-x</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>29019000</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Maternal and Child Health Journal</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Zhao</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>theimpactofnegativechildbirthexperienceonfuturereproductivedecisionsaquantitativesystematicreview2018shorey</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>the impact of negative childbirth experience on future reproductive decisions: a quantitative systematic review</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Shorey, Shefaly;Yang, Yen, Yen;Ang, Emily</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Aim: The aim of this study was to systematically retrieve, critique and synthesize available evidence regarding the association between negative childbirth experiences and future reproductive decisions. Background: A child's birth is often a joyous event; however, there is a proportion of women who undergo negative childbirth experiences that have long-term implications on their reproductive decisions. Design: A systematic review of quantitative studies was undertaken using Joanna Briggs Institute's methods. Review methods: A search was carried out in CINAHL Plus with Full Text, Embase, PsycINFO, PubMed, Scopus and Web of Science from January 1996-July 2016. Studies that fulfilled the inclusion criteria were assessed by two independent reviewers using the Joanna Briggs Institute's Critical Appraisal Tools. Data were extracted under subheadings adapted from the institute's data extraction forms. Results: Twelve studies, which examined either one or more influences of negative childbirth experiences, were identified. The included studies were either cohort or cross-sectional designs. Five studies observed positive associations between prior negative childbirth experiences and decisions to not have another child, three studies found positive associations between negative childbirth experiences and decisions to delay a subsequent birth and six studies concluded positive associations between negative childbirth experiences and maternal requests for caesarean section in subsequent pregnancies. Conclusion: To receive a holistic understanding on negative childbirth experiences, a suitable definition and validated measuring tools should be used to understand this phenomenon. Future studies or reviews should include a qualitative component and/or the exploration of specific factors such as cultural and regional differences that influence childbirth experiences. (PsycINFO Database Record (c) 2019 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>10.1111/jan.13534</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>29394456</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Journal of Advanced Nursing</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Shorey</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>feedingneonatesbycupasystematicreviewoftheliterature2016mckinney</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>feeding neonates by cup: a systematic review of the literature</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>McKinney, Christy, M.;Glass, Robin, P.;Coffey, Patricia;Rue, Tessa;Vaughn, Matthew, G.;Cunningham, Michael</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Objective: WHO and UNICEF recommend cup feeding for neonates unable to breastfeed in low-resource settings. In developed countries, cup feeding in lieu of bottle feeding in the neonatal period is hypothesized to improve breastfeeding outcomes for those initially unable to breastfeed. Our aim was to synthesize the entire body of evidence on cup feeding. Methods: We searched domestic and international databases for original research. Our search criteria required original data on cup feeding in neonates published in English between January 1990 and December 2014. Results: We identified 28 original research papers. Ten were randomized clinical trials, 7 non-randomized intervention studies, and 11 observational studies; 11 were conducted in developing country. Outcomes evaluated included physiologic stability, safety, intake, duration, spillage, weight gain, any and exclusive breastfeeding, length of hospital stay, compliance, and acceptability. Cup feeding appears to be safe though intake may be less and spillage greater relative to bottle or tube feeding. Overall, slightly higher proportions of cup fed versus bottle fed infants report any breastfeeding; a greater proportion of cup fed infants reported exclusive breastfeeding at discharge and beyond. Cup feeding increases breastfeeding in subgroups (e.g. those who intend to breastfeed or women who had a Caesarean section). Compliance and acceptability is problematic in certain settings. Conclusions: Further research on long-term breastfeeding outcomes and in low-resource settings would be helpful. Research data on high risk infants (e.g. those with cleft palates) would be informative. Innovative cup feeding approaches to minimize spillage, optimize compliance, and increase breastfeeding feeding are needed. (PsycINFO Database Record (c) 2017 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>10.1007/s10995-016-1961-9</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Maternal and Child Health Journal</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>McKinney</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>birthrelatedperinealtraumainlowandmiddleincomecountriesasystematicreviewandmetaanalysis2019aguiar</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>birth-related perineal trauma in low- and middle-income countries: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Aguiar, Magda;Farley, Amanda;Hope, Lucy;Amin, Adeela;Shah, Pooja;Manaseki-Holland, Semira</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Introduction: Birth-related perineal trauma (BPT) is a common consequence of vaginal births. When poorly managed, BPT can result in increased morbidity and mortality due to infections, haemorrhage, and incontinence. This review aims to collect data on rates of BPT in low- and middle-income countries (LMICs), through a systematic review and meta-analysis. Methods: The following databases were searched: Medline, Embase, Latin American and Caribbean Health Sciences Literature (LILACs), and the World Health Organization (WHO) regional databases, from 2004 to 2016. Cross-sectional data on the proportion of vaginal births that resulted in episiotomy, second degree tears or obstetric anal sphincter injuries (OASI) were extracted from studies carried out in LMICs by two independent reviewers. Estimates were meta-analysed using a random effects model; results were presented by type of BPT, parity, and mode of birth. Results: Of the 1182 citations reviewed, 74 studies providing data on 334,054 births in 41 countries were included. Five studies reported outcomes of births in the community. In LMICs, the overall rates of BPT were 46% (95% CI 36-55%), 24% (95% CI 17-32%), and 1.4% (95% CI 1.2-1.7%) for episiotomies, second degree tears, and OASI, respectively. Studies were highly heterogeneous with respect to study design and population. The overall reporting quality was inadequate. Discussion: Compared to high-income settings, episiotomy rates are high in LMIC medical facilities. There is an urgent need to improve reporting of BPT in LMICs particularly with regards to births taking in community settings. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>10.1007/s10995-019-02732-5</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>30915627</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Maternal and Child Health Journal</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Aguiar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>epilepsyinpregnancyandreproductiveoutcomesasystematicreviewandmetaanalysis2015viale</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>epilepsy in pregnancy and reproductive outcomes: a systematic review and meta-analysis</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Viale, Luz;Allotey, John;Cheong-See, Fiona;Arroyo-Manzano, David;Mccorry, Dougall;Bagary, Manny;Mignini, Luciano;Khan, Khalid, S;Zamora, Javier;Thangaratinam, Shakila</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Background: Antenatal care of women with epilepsy is varied. The association of epilepsy and antiepileptic drug exposure with pregnancy outcomes needs to be quantified to guide management. We did a systematic review and meta-analysis to investigate the association between epilepsy and reproductive outcomes, with or without exposure to antiepileptic drugs. Methods: We searched MEDLINE, Embase, Cochrane, AMED, and CINAHL between Jan 1, 1990, and Jan 21, 2015, with no language or regional restrictions, for observational studies of pregnant women with epilepsy, which assessed the risk of obstetric complications in the antenatal, intrapartum, or postnatal period, and any neonatal complications. We used the Newcastle-Ottawa Scale to assess the methodological quality of the included studies, risk of bias in the selection and comparability of cohorts, and outcome. We assessed the odds of maternal and fetal complications (excluding congenital malformations) by comparing pregnant women with and without epilepsy and undertook subgroup analysis based on antiepileptic drug exposure in women with epilepsy. We summarised the association as odds ratio (OR; 95% CI) using random effects meta-analysis. The PROSPERO ID of this Systematic Review's protocol is CRD42014007547. Findings: Of 7050 citations identified, 38 studies from low-income and high-income countries met our inclusion criteria (39 articles including 2 837 325 pregnancies). Women with epilepsy versus those without (2 809 984 pregnancies) had increased odds of spontaneous miscarriage (OR 1*54, 95% CI 1*02-2*32; I2 = 67%), antepartum haemorrhage (1*49, 1*01-2*20; I2 = 37%), post-partum haemorrhage (1*29, 1*13-1*49; I2 = 41%), hypertensive disorders (1*37, 1*21-1*55; I2 = 23%), induction of labour (1*67, 1*31-2*11; I2 = 64%), caesarean section (1*40, 1*23-1*58; I2 = 66%), any preterm birth (&lt;37 weeks of gestation; 1*16, 1*01-1*34; I2 = 64%), and fetal growth restriction (1*26, 1*20-1*33; I2 = 1%). The odds of early preterm birth, gestational diabetes, fetal death or stillbirth, perinatal death, or admission to neonatal intensive care unit did not differ between women with epilepsy and those without the disorder. Interpretation: A small but significant association of epilepsy, exposure to antiepileptic drugs, and adverse outcomes exists in pregnancy. This increased risk should be taken into account when counselling women with epilepsy. Funding: EBM CONNECT Collaboration. (PsycINFO Database Record (c) 2016 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>10.1016/S0140-6736(15)00045-8</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>26318519</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>The Lancet</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Viale</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>cesareansectionandriskofpostpartumdepressionametaanalysis2017xu</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>cesarean section and risk of postpartum depression: a meta-analysis</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Xu, Hui;Ding, Yu;Ma, Yue;Xin, Xueling;Zhang, Dongfeng</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Objective: The association of cesarean section (CS) with the risk of postpartum depression (PPD) remains controversial. Therefore, we conducted a meta-analysis to explore the association between CS and the risk of PPD. Methods: A systematic literature search was performed in PubMed, Web of Science and Embase databases for relevant articles up to November 2016. Pooled odds ratios (ORs) with 95% confidence intervals (CIs) were calculated with fixed-effects model or random-effects model. Results: A total of 28 studies from 27 articles involving 532,630 participants were included in this meta-analysis. The pooled OR of the association between CS and PPD risk was 1.26 (95% CI: 1.16-1.36). In subgroup analyses stratified by study design [cohort studies: (1.25, 95% CI: 1.10-1.41); case-control studies: (1.25, 95% CI: 1.00-1.56); cross-sectional studies: (1.44, 95% CI: 1.14-1.82)] and adjustment status of complications during pregnancy [adjusted for: (1.29, 95% CI: 1.12-1.48); not-adjusted for: (1.24, 95% CI: 1.13-1.36)], the abovementioned associations remained consistent. The pooled ORs of PPD were 1.15 (95% CI: 0.92-1.43) for elective cesarean section (ElCS) and 1.47 (95% CI: 1.33-1.62) for emergency cesarean section (EmCS). Conclusion: This meta-analysis suggests that CS and EmCS increase the risk of PPD. Further evidence is needed to explore the associations between the specific types of CS and the risk of PPD. (PsycInfo Database Record (c) 2020 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>10.1016/j.jpsychores.2017.04.016</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>28606491</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Journal of Psychosomatic Research</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Xu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>genderandbirthcohortdifferencesinadultattachmentinchinesecollegestudentsametaanalysis2017shu</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>gender and birth cohort differences in adult attachment in chinese college students: a meta-analysis</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Shu, Cong;Chen, Xu;Liu, Ying;Zhang, Xing;Hu, Dengyu;Hu, Na;Liu, Xinyi</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Since China adopted its reform and opening-up policy, the state of society has changed dramatically. Correspondingly, Chinese college students' scores of the Experiences in Close Relationships scale are expected to have changed from 2003 to 2015. A cross-temporal meta-analysis found that Chinese college students' scores of the attachment anxiety subscale increased by 0.2 standard deviations in the past 13years. With a turning point in 2009, the scores of the attachment avoidance subscale increased by 0.58 standard deviations from 2003 to 2009 and decreased by 0.57 standard deviations from 2009 to 2015. Five social indicators including divorce rate, C-section rate, household size, Consumer Price Index, and Gini coefficient showed significant correlation with attachment anxiety. The results from a second meta-analysis showed that there was no gender difference or cohort effect in gender difference in Chinese college students' adult attachment scores. Finally, the explanations and implications of these changes and the insignificant gender difference are discussed. (PsycInfo Database Record (c) 2020 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>10.1016/j.paid.2016.10.012</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Personality and Individual Differences</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Shu</t>
         </is>
       </c>
     </row>
@@ -4931,7 +4932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4993,120 +4994,6 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>first_author_surname</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>pentobarbitalcomauseinapregnantpatientwithrefractoryintracranialhypertension:acasereport;2022;patel</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>pentobarbital coma use in a pregnant patient with refractory intracranial hypertension: a case report</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Patel, Devan;Dehne, Kelly;Pajer, Hengameh;Barnett, Randaline;Sasaki-Adams, Deanna;Quinsey, Carolyn</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Objective: Intracranial hypertension is a life-threatening condition that requires emergent diagnosis and management. Although pentobarbital coma for refractory intracranial hypertension has been studied in the general population, this study is the first reported case of pentobarbital coma use in a pregnant patient. Methods: We performed a retrospective chart review of a pregnant patient with refractory intracranial hypertension and reviewed the current literature on the role of pentobarbital coma. Results: We present the case of a 35-year-old woman at 26 weeks of gestation who developed refractory intracranial hypertension secondary to rupture of a dural arteriovenous fistula. The patient was taken to surgery for decompressive hemicraniectomy, clot evacuation, and dural arteriovenous fistula resection. Subsequently, the patient was treated with pentobarbital coma for 5 days and achieved adequate control of her intracranial pressures. The patient and fetus were closely monitored by the obstetrics team with no apparent harm to fetal well-being during her hospital stay. The patient underwent planned cesarean delivery at term, and both the mother and newborn were discharged in stable condition with no known pentobarbital-related complications. Conclusions: Thus, we present the first case report demonstrating that pentobarbital coma may be a safe and efficacious option for treating pregnant patients with life-threatening refractory intracranial hypertension. We also provide dosing information for pentobarbital administration. Additional studies and reports involving pregnant patients are needed to better understand the impact of pentobarbital on both the mother and fetus. Furthermore, long-term follow-up of both the mother and newborn is critical to identifying any delayed sequelae of neonatal exposure to pentobarbital. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>10.1097/WNF.0000000000000496</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>35195548</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Clinical Neuropharmacology</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Patel</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>potentialofgeographicalvariationanalysisforrealigningproviderstovalue-basedcare.echocasestudyonlower-valueindicationsofc-sectioninfiveeuropeancountries;2015;garcia-armesto</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>potential of geographical variation analysis for realigning providers to value-based care. echo case study on lower-value indications of c-section in five european countries</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>2015</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Garcia-Armesto, Sandra;Angulo-Pueyo, Ester;Martinez-Lizaga, Natalia;Mateus, Ceu;Joaquim, Ines;Bernal-Delgado, Enrique</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Background: Although C-section is a highly effective procedure, literature abounds with evidence of overuse and particularly misuse, in lower-value indications such as low-risk deliveries. This study aims to quantify utilization of C-section in low-risk cases, mapping out areas showing excess-usage in each country and to estimate excess-expenditure as a proxy of the opportunity cost borne by healthcare systems. Methods: Observational, ecologic study on deliveries in 913 sub-national administrative areas of five European countries (Denmark, England, Portugal, Slovenia and Spain) from 2002 to 2009. The study includes a cross-section analysis with 2009 data and a time-trend analysis for the whole period. Main endpoints: age-standardized utilization rates of C-section in low-risk pregnancies and deliveries per 100 deliveries. Secondary endpoints: Estimated excess-cases per geographical unit of analysis in two scenarios of minimized utilization. Results: C-section is widely used in all examined countries (ranging from 19% of Slovenian deliveries to 33% of deliveries in Portugal). With the exception of Portugal, there are no systematic variations in intensity of use across areas in the same country. Cross-country comparison of lower-value C-section leaves Denmark with 10% and Portugal with 2%, the highest and lowest. Such behaviour was stable over the period of analysis. Within each country, the scattered geographical patterns of use intensity speak for local drivers playing a major role within the national trend. Conclusion: The analysis conducted suggests plenty of room for enhancing value in obstetric care and equity in women's access to such within the countries studied. The analysis of geographical variations in lower-value care can constitute a powerful screening tool. (PsycINFO Database Record (c) 2016 APA, all rights reserved)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>10.1093/eurpub/cku224</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>European Journal of Public Health</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Peer Reviewed Journal</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Journal Article;</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>English</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Garcia-Armesto</t>
         </is>
       </c>
     </row>
@@ -5116,6 +5003,196 @@
 </file>
 
 <file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dedup_index</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>authors</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>abstract</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>doi</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>pmid</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>journal</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>pubtype</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>publication types</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>first_author_surname</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>pentobarbitalcomauseinapregnantpatientwithrefractoryintracranialhypertensionacasereport2022patel</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>pentobarbital coma use in a pregnant patient with refractory intracranial hypertension: a case report</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Patel, Devan;Dehne, Kelly;Pajer, Hengameh;Barnett, Randaline;Sasaki-Adams, Deanna;Quinsey, Carolyn</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Objective: Intracranial hypertension is a life-threatening condition that requires emergent diagnosis and management. Although pentobarbital coma for refractory intracranial hypertension has been studied in the general population, this study is the first reported case of pentobarbital coma use in a pregnant patient. Methods: We performed a retrospective chart review of a pregnant patient with refractory intracranial hypertension and reviewed the current literature on the role of pentobarbital coma. Results: We present the case of a 35-year-old woman at 26 weeks of gestation who developed refractory intracranial hypertension secondary to rupture of a dural arteriovenous fistula. The patient was taken to surgery for decompressive hemicraniectomy, clot evacuation, and dural arteriovenous fistula resection. Subsequently, the patient was treated with pentobarbital coma for 5 days and achieved adequate control of her intracranial pressures. The patient and fetus were closely monitored by the obstetrics team with no apparent harm to fetal well-being during her hospital stay. The patient underwent planned cesarean delivery at term, and both the mother and newborn were discharged in stable condition with no known pentobarbital-related complications. Conclusions: Thus, we present the first case report demonstrating that pentobarbital coma may be a safe and efficacious option for treating pregnant patients with life-threatening refractory intracranial hypertension. We also provide dosing information for pentobarbital administration. Additional studies and reports involving pregnant patients are needed to better understand the impact of pentobarbital on both the mother and fetus. Furthermore, long-term follow-up of both the mother and newborn is critical to identifying any delayed sequelae of neonatal exposure to pentobarbital. (PsycInfo Database Record (c) 2022 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10.1097/WNF.0000000000000496</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>35195548</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Clinical Neuropharmacology</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Patel</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>potentialofgeographicalvariationanalysisforrealigningproviderstovaluebasedcareechocasestudyonlowervalueindicationsofcsectioninfiveeuropeancountries2015garciaarmesto</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>potential of geographical variation analysis for realigning providers to value-based care. echo case study on lower-value indications of c-section in five european countries</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2015</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Garcia-Armesto, Sandra;Angulo-Pueyo, Ester;Martinez-Lizaga, Natalia;Mateus, Ceu;Joaquim, Ines;Bernal-Delgado, Enrique</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Background: Although C-section is a highly effective procedure, literature abounds with evidence of overuse and particularly misuse, in lower-value indications such as low-risk deliveries. This study aims to quantify utilization of C-section in low-risk cases, mapping out areas showing excess-usage in each country and to estimate excess-expenditure as a proxy of the opportunity cost borne by healthcare systems. Methods: Observational, ecologic study on deliveries in 913 sub-national administrative areas of five European countries (Denmark, England, Portugal, Slovenia and Spain) from 2002 to 2009. The study includes a cross-section analysis with 2009 data and a time-trend analysis for the whole period. Main endpoints: age-standardized utilization rates of C-section in low-risk pregnancies and deliveries per 100 deliveries. Secondary endpoints: Estimated excess-cases per geographical unit of analysis in two scenarios of minimized utilization. Results: C-section is widely used in all examined countries (ranging from 19% of Slovenian deliveries to 33% of deliveries in Portugal). With the exception of Portugal, there are no systematic variations in intensity of use across areas in the same country. Cross-country comparison of lower-value C-section leaves Denmark with 10% and Portugal with 2%, the highest and lowest. Such behaviour was stable over the period of analysis. Within each country, the scattered geographical patterns of use intensity speak for local drivers playing a major role within the national trend. Conclusion: The analysis conducted suggests plenty of room for enhancing value in obstetric care and equity in women's access to such within the countries studied. The analysis of geographical variations in lower-value care can constitute a powerful screening tool. (PsycINFO Database Record (c) 2016 APA, all rights reserved)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>10.1093/eurpub/cku224</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>European Journal of Public Health</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Peer Reviewed Journal</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Journal Article;</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Garcia-Armesto</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5645,7 +5722,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>usinggradeasaframeworktoguideresearchonthesexualandreproductivehealthandrights(srhr)ofwomenlivingwithhiv--methodologicalopportunitiesandchallenges;2017;siegfried</t>
+          <t>usinggradeasaframeworktoguideresearchonthesexualandreproductivehealthandrightssrhrofwomenlivingwithhivmethodologicalopportunitiesandchallenges2017siegfried</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>